<commit_message>
qa-runs: apply UI-driven Kroki + explicit label to wyszukiwarka-instytucji run
- Kroki dla 10 cases przepisane na UI-driven (Otworz base URL -> akcje w UI):
  INST-01, 02, 03, 04, 05, 06, 11, 13, 14, 16. Tester nie musi konstruowac
  URL-i z query params, tylko klikac/wpisywac zgodnie z krokami.
- INST-07 i INST-19 zostaja URL-driven z notatka wyjatku:
  - INST-07: "URL jest przedmiotem testu (deep-link + param injection)"
  - INST-19: "URL jako skrot do stanu 'ostatnia strona'; interakcja Next
    pokryta w INST-17"
- Explicit label w Dane testowe dla INST-01 (frazy) i INST-10 (miejscowosci);
  kroki referencuja przez "wpisz fraze z Dane testowe ('val')".
- Consistency: zdjete ?limit=20&offset=0 z kroku 1 w INST-08/09/12
  (bazowy URL bez params zgodnie z regula UI-driven).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
+++ b/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
@@ -627,7 +627,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">fraza: </t>
+            <t xml:space="preserve">fraza używana w krokach: </t>
           </r>
           <r>
             <rPr>
@@ -642,6 +642,21 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
+            <t xml:space="preserve">; alternatywy do exploratory: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Warszawa"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
             <t xml:space="preserve">, </t>
           </r>
           <r>
@@ -650,21 +665,6 @@
               <b val="1"/>
               <sz val="10"/>
             </rPr>
-            <t>"Warszawa"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">, </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
             <t>"AGH"</t>
           </r>
         </is>
@@ -685,7 +685,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0&amp;search=Vistula</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -693,7 +693,38 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Poczekaj ~2s na render listy</t>
+2) W pole wyszukiwania z placeholderem </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Nazwa, fragment nazwy"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> wpisz frazę z Dane testowe (</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Vistula"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t>)
+3) Poczekaj ~2–3s na debounce i odświeżenie listy</t>
           </r>
         </is>
       </c>
@@ -824,7 +855,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0&amp;search=Vistula</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -832,7 +863,39 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Zbadaj atrybut target linku pierwszej instytucji w tabeli</t>
+2) W pole wyszukiwania wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Vistula"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i poczekaj ~2–3s na odświeżenie listy
+3) Kliknij nazwę pierwszej instytucji w tabeli wyników (link </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Akademia Finansów i Biznesu Vistula"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t>)
+4) Sprawdź czy strona detali otworzyła się w nowej karcie przeglądarki</t>
           </r>
         </is>
       </c>
@@ -978,7 +1041,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/instytucje/Akademia-Finans%C3%B3w-i-Biznesu-Vistula,30170</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -986,7 +1049,39 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Zlokalizuj sekcję </t>
+2) W pole wyszukiwania wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Vistula"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i poczekaj na odświeżenie listy
+3) Kliknij nazwę </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Akademia Finansów i Biznesu Vistula"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (otwiera się nowa karta)
+4) Na stronie detali zlokalizuj sekcję </t>
           </r>
           <r>
             <rPr>
@@ -1002,7 +1097,22 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-3) Zbadaj atrybuty target i rel linku zewnętrznego</t>
+5) Kliknij link </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"http://www.vistula.edu.pl"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i sprawdź czy otwiera się w nowej karcie</t>
           </r>
         </is>
       </c>
@@ -1118,7 +1228,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0&amp;search=</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -1126,7 +1236,40 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Poczekaj ~2s</t>
+2) W pole wyszukiwania wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Vistula"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i poczekaj aż licznik spadnie do 22
+3) Zaznacz całą frazę w polu (Cmd</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="FF0563C1"/>
+              <sz val="10"/>
+              <u val="single"/>
+            </rPr>
+            <t>/Ctrl</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t>+A) i naciśnij Delete żeby wyczyścić
+4) Poczekaj ~2–3s na odświeżenie listy</t>
           </r>
         </is>
       </c>
@@ -1234,7 +1377,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0&amp;search=nieistniejacax9y9z9qwerty</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -1242,7 +1385,23 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Poczekaj ~2s</t>
+2) W pole wyszukiwania wpisz frazę </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"nieistniejacax9y9z9qwerty"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+3) Poczekaj ~2–3s na odświeżenie listy</t>
           </r>
         </is>
       </c>
@@ -1433,11 +1592,118 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>1) Otwórz ?search=łódź (URL-encoded)
-2) Zapisz licznik (spodziewane 84)
-3) Otwórz ?search=ŁÓDŹ i porównaj licznik z krokiem 2
-4) Otwórz ?search=%20%20Vistula%20%20 i sprawdź czy licznik = ?search=Vistula (22)
-5) Otwórz ?search=Filia; i sprawdź &gt;0 wyników z semikolonem w nazwach</t>
+            <t xml:space="preserve">1) Otwórz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="FF0563C1"/>
+              <sz val="10"/>
+              <u val="single"/>
+            </rPr>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+2) W pole wyszukiwania wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"łódź"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (małe litery, z polskimi znakami), poczekaj ~3s, zapisz licznik (spodziewane 84)
+3) Wyczyść pole (Cmd</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="FF0563C1"/>
+              <sz val="10"/>
+              <u val="single"/>
+            </rPr>
+            <t>/Ctrl</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">+A + Delete), wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"ŁÓDŹ"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (wielkie litery), poczekaj i porównaj licznik z krokiem 2
+4) Wyczyść, wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"  Vistula  "</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (2 spacje przed i po), poczekaj, sprawdź czy licznik = 22 (jak dla </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Vistula"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> bez spacji)
+5) Wyczyść, wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Filia;"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (ze średnikiem), poczekaj, sprawdź licznik &gt;0</t>
           </r>
         </is>
       </c>
@@ -1574,9 +1840,56 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>1) Otwórz ?search=aaa…(500 znaków) i sprawdź brak crashu
-2) Otwórz ?search=%3Cscript%3Ealert(1)%3C%2Fscript%3E&amp;limit=abc&amp;offset=-1
-3) Sprawdź czy nie pojawia się dialog alert, brak &lt;script&gt; w DOM, licznik = 0</t>
+            <t xml:space="preserve">1) Otwórz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="FF0563C1"/>
+              <sz val="10"/>
+              <u val="single"/>
+            </rPr>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0&amp;search=aaa…(500</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> znaków </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"a"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">) — sprawdź brak crashu, licznik = 0
+2) Otwórz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="FF0563C1"/>
+              <sz val="10"/>
+              <u val="single"/>
+            </rPr>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=abc&amp;offset=-1&amp;search=%3Cscript%3Ealert(1</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t>)%3C%2Fscript%3E
+3) Sprawdź czy nie pojawia się dialog alert, brak &lt;script&gt; w DOM, payload wyrenderowany jako tekst w polu wyszukiwania</t>
           </r>
         </is>
       </c>
@@ -1619,7 +1932,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>500-char query: 0 wyników, ""Brak danych"", brak crashu. XSS: script jako tekst w polu, brak execution. Widget normalizował limit=abc→20; offset=-1 przekonwertowany na -20 (dziwne, ale bez crashu)</t>
+          <t>URL jest przedmiotem testu (deep-link + param injection) — kroki URL-driven są celowe. 500-char query: 0 wyników, ""Brak danych"", brak crashu. XSS: script jako tekst w polu, brak execution. Widget normalizował limit=abc→20; offset=-1 przekonwertowany na -20 (dziwne, ale bez crashu)</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1998,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -1693,7 +2006,22 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Zaznacz checkbox </t>
+2) W sekcji filtrów </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Zadania w ZSK"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> zaznacz checkbox </t>
           </r>
           <r>
             <rPr>
@@ -1702,21 +2030,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Instytucja certyfikująca (IC)"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> w sekcji </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Zadania w ZSK"</t>
           </r>
         </is>
       </c>
@@ -1847,7 +2160,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -1855,7 +2168,37 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Zaznacz checkbox </t>
+2) W sekcji filtrów </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Kategoria kwalifikacji"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (grupa </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Edukacja pozaformalna"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">) zaznacz checkbox </t>
           </r>
           <r>
             <rPr>
@@ -1864,21 +2207,6 @@
               <sz val="10"/>
             </rPr>
             <t>"wolnorynkowe"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> w sekcji </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Kategoria kwalifikacji"</t>
           </r>
         </is>
       </c>
@@ -1958,7 +2286,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">miejscowość: </t>
+            <t xml:space="preserve">miejscowość używana w krokach: </t>
           </r>
           <r>
             <rPr>
@@ -1973,7 +2301,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">, inne: </t>
+            <t xml:space="preserve">; alternatywy do exploratory: </t>
           </r>
           <r>
             <rPr>
@@ -2031,7 +2359,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -2054,8 +2382,23 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve"> w sekcji Siedziba
-3) Wpisz min. 3 znaki: </t>
+            <t xml:space="preserve"> w sekcji </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Siedziba instytucji certyfikującej"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+3) Wpisz min. 3 znaki miejscowości z Dane testowe (</t>
           </r>
           <r>
             <rPr>
@@ -2070,8 +2413,8 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">
-4) Wybierz opcję </t>
+            <t>)
+4) Z listy podpowiedzi wybierz odpowiednią opcję (</t>
           </r>
           <r>
             <rPr>
@@ -2086,7 +2429,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve"> z listy podpowiedzi</t>
+            <t>)</t>
           </r>
         </is>
       </c>
@@ -2186,7 +2529,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0&amp;roles=1&amp;qualification_categories=5</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -2194,7 +2537,69 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Poczekaj na wynik</t>
+2) W sekcji filtrów </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Zadania w ZSK"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> zaznacz checkbox </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Instytucja certyfikująca (IC)"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">, zapisz licznik (~579)
+3) W sekcji </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Kategoria kwalifikacji"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> zaznacz checkbox </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"wolnorynkowe"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+4) Poczekaj na odświeżenie listy i sprawdź licznik po kombinacji</t>
           </r>
         </is>
       </c>
@@ -2310,7 +2715,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -2318,7 +2723,7 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Kliknij ikonę informacji (i) obok nagłówka </t>
+2) Kliknij ikonę informacji (i) obok nagłówka filtra </t>
           </r>
           <r>
             <rPr>
@@ -2472,7 +2877,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0&amp;roles=1&amp;search=nieistniejaca_instytucja_xyz</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -2480,7 +2885,54 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Poczekaj ~2s</t>
+2) W sekcji </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Zadania w ZSK"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> zaznacz checkbox </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Instytucja certyfikująca (IC)"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+3) W pole wyszukiwania wpisz frazę </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"nieistniejaca_instytucja_xyz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+4) Poczekaj ~2–3s na odświeżenie listy</t>
           </r>
         </is>
       </c>
@@ -2596,7 +3048,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0&amp;search=Vistula</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -2604,7 +3056,23 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Kliknij przycisk </t>
+2) W pole wyszukiwania wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Vistula"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i poczekaj aż licznik spadnie do 22
+3) Kliknij przycisk </t>
           </r>
           <r>
             <rPr>
@@ -2620,7 +3088,7 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve"> w prawym górnym rogu listy
-3) Sprawdź liczbę wierszy w pobranym pliku</t>
+4) Otwórz pobrany plik i sprawdź liczbę wierszy</t>
           </r>
         </is>
       </c>
@@ -2844,7 +3312,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0&amp;search=nieistniejaca_xyz</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -2852,7 +3320,38 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Kliknij </t>
+2) W pole wyszukiwania wpisz frazę </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"nieistniejaca_xyz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i poczekaj aż licznik pokaże </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Znaleziono: 0"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+3) Kliknij przycisk </t>
           </r>
           <r>
             <rPr>
@@ -2868,7 +3367,7 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-3) Sprawdź zawartość pobranego pliku</t>
+4) Otwórz pobrany plik i sprawdź czy zawiera nagłówek kolumn</t>
           </r>
         </is>
       </c>
@@ -3357,9 +3856,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>URL ?offset=2600 jako skrót do stanu „ostatnia strona"; interakcja Next pokryta w INST-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
qa-runs: apply "testowania manualnego" replacement to wyszukiwarka-instytucji
INST-01 i INST-10 (cases z alternatywnymi wartosciami w Dane testowe):
"alternatywy do exploratory" -> "alternatywy do testowania manualnego".
XLSX zregenerowany.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
+++ b/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
@@ -645,7 +645,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">; alternatywy do exploratory: </t>
+            <t xml:space="preserve">; alternatywy do testowania manualnego: </t>
           </r>
           <r>
             <rPr>
@@ -2585,7 +2585,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">; alternatywy do exploratory: </t>
+            <t xml:space="preserve">; alternatywy do testowania manualnego: </t>
           </r>
           <r>
             <rPr>

</xml_diff>

<commit_message>
qa-runs: remove out-of-scope "(case-insensitive)" + translate remaining jargon
INST-01 Expected: usuniete "(case-insensitive)" — case testuje fakt zwrocenia
wynikow dla frazy "Vistula", nie sprawdza wielkosci liter. Case-insensitivity
jest dedicated w INST-06. Uwaga poza scope zmyla testera.

INST-06 Notatki + report ("Rzeczywisty rezultat"):
- "case-insensitive" -> "wielkosc liter ignorowana"
- "trim" -> "przycinanie spacji na krancach"
- "Bundle 4 patterns w 1 edge case" -> "4 warianty input w jednym przypadku
  brzegowym"
- "semikolon" -> "srednik", "query" -> "wyszukiwanie"
- Notatka INST-06 przepisana z developerskiego skrotu ("Trim spacji ✓, ...")
  na pelne PL zdanie.

XLSX zregenerowany.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
+++ b/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
@@ -769,7 +769,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" (case-insensitive)</t>
+            <t>""</t>
           </r>
         </is>
       </c>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
-          <t>Trim spacji ✓, case-insensitive PL ✓, semikolon w query ✓. Bundle 4 patterns w 1 edge case</t>
+          <t>Sprawdzone: przycinanie spacji na krańcach, ignorowanie wielkości liter dla polskich znaków, średnik jako znak specjalny nie łamie wyszukiwania. 4 warianty input w jednym przypadku brzegowym</t>
         </is>
       </c>
     </row>
@@ -5368,7 +5368,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>łódź=84, ŁÓDŹ=84 (case-insensitive); "</t>
+            <t>łódź=84, ŁÓDŹ=84 (wielkość liter ignorowana); "</t>
           </r>
           <r>
             <rPr>
@@ -5383,7 +5383,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" (z spacjami) = Vistula = 22 (trim); Filia; = 204 (semikolon jako znak specjalny nie łamie query)</t>
+            <t>" (z spacjami) = Vistula = 22 (spacje na krańcach przycięte); Filia; = 204 (średnik jako znak specjalny nie łamie wyszukiwania)</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
qa-runs: generate bug reports for wyszukiwarka-instytucji FAIL cases
Applied new bug-reports feature retroactively to current run.

Nowe artefakty:
- wyszukiwarka-instytucji-2026-08-15-bugs.tsv (15 kolumn: Priorytet +
  Waznosc + structured Srodowisko + 4 sekcje)
- bugs/INST-BR-01.md (asciifolding — Priorytet P2 Wysoki, Waznosc Medium)
- bugs/INST-BR-02.md (empty download — Priorytet P3 Niski, Waznosc Low)

XLSX ma teraz 4 zakladki: Test cases · Execution report · INST-BR-01
(zolty tab Medium) · INST-BR-02 (szary tab Low).

Zmiany w istniejacych plikach:
- cases.tsv, report.tsv, .md: INST-BR-03 -> INST-BR-02 (renumbering, zeby
  bugi byly sekwencyjne 01/02)
- report.tsv Reprodukcja + .md report block: zsynchronizowana z case's
  Kroki dla FAIL rows (UI-driven, spojnosc miedzy cases/report/bugs)
- XLSX zregenerowany

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
+++ b/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution report" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INST-BR-01" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INST-BR-02" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +43,26 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00305496"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +109,11 @@
         <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -116,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -162,6 +187,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -738,7 +775,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Licznik "</t>
+            <t xml:space="preserve">Licznik </t>
           </r>
           <r>
             <rPr>
@@ -751,10 +788,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" pokazuje wartość &gt;0 a nazwy w wierszach zawierają frazę "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> pokazuje wartość &gt;0 a nazwy w wierszach zawierają frazę </t>
           </r>
           <r>
             <rPr>
@@ -763,13 +799,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Vistula"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>""</t>
           </r>
         </is>
       </c>
@@ -823,7 +852,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>pierwszy wiersz w tabeli (link "</t>
+            <t xml:space="preserve">pierwszy wiersz w tabeli (link </t>
           </r>
           <r>
             <rPr>
@@ -838,7 +867,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>")</t>
+            <t>)</t>
           </r>
         </is>
       </c>
@@ -909,7 +938,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Link do detalu ma target="</t>
+            <t>Link do detalu ma target=</t>
           </r>
           <r>
             <rPr>
@@ -924,7 +953,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">" i wskazuje na </t>
+            <t xml:space="preserve"> i wskazuje na </t>
           </r>
           <r>
             <rPr>
@@ -983,7 +1012,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Otwarta strona szczegółów instytucji z sekcją "</t>
+            <t xml:space="preserve">Otwarta strona szczegółów instytucji z sekcją </t>
           </r>
           <r>
             <rPr>
@@ -993,13 +1022,6 @@
             </rPr>
             <t>"Zobacz stronę instytucji"</t>
           </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
-          </r>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -1009,7 +1031,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>link "</t>
+            <t xml:space="preserve">link </t>
           </r>
           <r>
             <rPr>
@@ -1024,7 +1046,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" na profilu Akademia Finansów i Biznesu Vistula</t>
+            <t xml:space="preserve"> na profilu Akademia Finansów i Biznesu Vistula</t>
           </r>
         </is>
       </c>
@@ -1126,7 +1148,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Link do strony instytucji ma target="</t>
+            <t>Link do strony instytucji ma target=</t>
           </r>
           <r>
             <rPr>
@@ -1139,10 +1161,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" oraz rel="</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> oraz rel=</t>
           </r>
           <r>
             <rPr>
@@ -1151,13 +1172,6 @@
               <sz val="10"/>
             </rPr>
             <t>"noopener noreferrer"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -1283,7 +1297,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Licznik "</t>
+            <t xml:space="preserve">Licznik </t>
           </r>
           <r>
             <rPr>
@@ -1298,7 +1312,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" (pełna lista), URL param search= jest ignorowany lub stripowany</t>
+            <t xml:space="preserve"> (pełna lista), URL param search= jest ignorowany lub stripowany</t>
           </r>
         </is>
       </c>
@@ -1415,7 +1429,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Licznik "</t>
+            <t xml:space="preserve">Licznik </t>
           </r>
           <r>
             <rPr>
@@ -1428,10 +1442,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>", tabela pokazuje wiersz "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">, tabela pokazuje wiersz </t>
           </r>
           <r>
             <rPr>
@@ -1440,13 +1453,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Brak danych"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -1489,7 +1495,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Baza zawiera instytucje z "</t>
+            <t xml:space="preserve">Baza zawiera instytucje z </t>
           </r>
           <r>
             <rPr>
@@ -1502,10 +1508,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" (~84) i "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (~84) i </t>
           </r>
           <r>
             <rPr>
@@ -1520,7 +1525,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" (~200) w nazwie</t>
+            <t xml:space="preserve"> (~200) w nazwie</t>
           </r>
         </is>
       </c>
@@ -1733,7 +1738,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>, znaki specjalne z dataset) zwracają oczekiwane liczby bez błędu: łódź=ŁÓDŹ=84, "</t>
+            <t xml:space="preserve">, znaki specjalne z dataset) zwracają oczekiwane liczby bez błędu: łódź=ŁÓDŹ=84, </t>
           </r>
           <r>
             <rPr>
@@ -1748,7 +1753,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>"=Vistula=22, Filia;=204</t>
+            <t>=Vistula=22, Filia;=204</t>
           </r>
         </is>
       </c>
@@ -1950,7 +1955,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Licznik dla "</t>
+            <t xml:space="preserve">Licznik dla </t>
           </r>
           <r>
             <rPr>
@@ -1963,10 +1968,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" ≈ licznik dla "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> ≈ licznik dla </t>
           </r>
           <r>
             <rPr>
@@ -1979,10 +1983,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" (~84); backend normalizuje diakrytyki (unaccent / asciifolding) i znajduje nazwy z "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (~84); backend normalizuje diakrytyki (unaccent / asciifolding) i znajduje nazwy z </t>
           </r>
           <r>
             <rPr>
@@ -1995,10 +1998,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" niezależnie od tego czy user wpisał "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> niezależnie od tego czy user wpisał </t>
           </r>
           <r>
             <rPr>
@@ -2011,10 +2013,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" czy "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> czy </t>
           </r>
           <r>
             <rPr>
@@ -2023,13 +2024,6 @@
               <sz val="10"/>
             </rPr>
             <t>"łódź"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -2216,7 +2210,7 @@
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>URL jest przedmiotem testu (deep-link + param injection) — kroki URL-driven są celowe. 500-char query: 0 wyników, ""Brak danych"", brak crashu. XSS: script jako tekst w polu, brak execution. Widget normalizował limit=abc→20; offset=-1 przekonwertowany na -20 (dziwne, ale bez crashu)</t>
+          <t>URL jest przedmiotem testu (deep-link + param injection) — kroki URL-driven są celowe. 500-char query: 0 wyników, "Brak danych", brak crashu. XSS: script jako tekst w polu, brak execution. Widget normalizował limit=abc→20; offset=-1 przekonwertowany na -20 (dziwne, ale bez crashu)</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2318,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Licznik "</t>
+            <t xml:space="preserve">Licznik </t>
           </r>
           <r>
             <rPr>
@@ -2337,10 +2331,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" spada z 2605 do &lt;2605, URL zawiera "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> spada z 2605 do &lt;2605, URL zawiera </t>
           </r>
           <r>
             <rPr>
@@ -2349,13 +2342,6 @@
               <sz val="10"/>
             </rPr>
             <t>"&amp;roles=1"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -2501,7 +2487,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Licznik spada z 2605 do &lt;2605, URL zawiera "</t>
+            <t xml:space="preserve">Licznik spada z 2605 do &lt;2605, URL zawiera </t>
           </r>
           <r>
             <rPr>
@@ -2510,13 +2496,6 @@
               <sz val="10"/>
             </rPr>
             <t>"&amp;qualification_categories=5"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -2724,7 +2703,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Licznik spada do &lt;2605, URL zawiera "</t>
+            <t xml:space="preserve">Licznik spada do &lt;2605, URL zawiera </t>
           </r>
           <r>
             <rPr>
@@ -2733,13 +2712,6 @@
               <sz val="10"/>
             </rPr>
             <t>"&amp;cities=Warszawa"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -2948,7 +2920,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>ikona (i) obok nagłówka "</t>
+            <t xml:space="preserve">ikona (i) obok nagłówka </t>
           </r>
           <r>
             <rPr>
@@ -2961,10 +2933,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" i "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i </t>
           </r>
           <r>
             <rPr>
@@ -2973,13 +2944,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Kategoria kwalifikacji"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -3026,7 +2990,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Otwiera się modal z nagłówkiem "</t>
+            <t xml:space="preserve">Otwiera się modal z nagłówkiem </t>
           </r>
           <r>
             <rPr>
@@ -3039,10 +3003,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" i treścią definicji (np. dla IC: "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i treścią definicji (np. dla IC: </t>
           </r>
           <r>
             <rPr>
@@ -3057,7 +3020,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>")</t>
+            <t>)</t>
           </r>
         </is>
       </c>
@@ -3073,7 +3036,7 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Ikona pomocy tylko dla 2 z 3 filtrów (brak dla ""Siedziba"" — pewnie by design)</t>
+          <t>Ikona pomocy tylko dla 2 z 3 filtrów (brak dla "Siedziba" — pewnie by design)</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3190,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Licznik "</t>
+            <t xml:space="preserve">Licznik </t>
           </r>
           <r>
             <rPr>
@@ -3240,10 +3203,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>", tabela "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">, tabela </t>
           </r>
           <r>
             <rPr>
@@ -3252,13 +3214,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Brak danych"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -3383,7 +3338,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Pobrany plik zawiera header + X wierszy danych (odpowiada widocznemu licznikowi "</t>
+            <t xml:space="preserve">Pobrany plik zawiera header + X wierszy danych (odpowiada widocznemu licznikowi </t>
           </r>
           <r>
             <rPr>
@@ -3398,7 +3353,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>"), format .xlsx</t>
+            <t>), format .xlsx</t>
           </r>
         </is>
       </c>
@@ -3662,7 +3617,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Przycisk "</t>
+            <t xml:space="preserve">Przycisk </t>
           </r>
           <r>
             <rPr>
@@ -3677,7 +3632,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" jest wyłączony LUB pobrany plik zawiera co najmniej nagłówek kolumn (nie tylko pusty arkusz)</t>
+            <t xml:space="preserve"> jest wyłączony LUB pobrany plik zawiera co najmniej nagłówek kolumn (nie tylko pusty arkusz)</t>
           </r>
         </is>
       </c>
@@ -3688,12 +3643,12 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>INST-BR-03</t>
+          <t>INST-BR-02</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Przycisk nie jest disabled, plik ma 1×1 arkusz z pustą komórką (brak nawet nagłówka ""#/ID/Nazwa"") — mylące dla usera</t>
+          <t>Przycisk nie jest disabled, plik ma 1×1 arkusz z pustą komórką (brak nawet nagłówka "#/ID/Nazwa") — mylące dla usera</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3686,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Kliknięcie "</t>
+            <t xml:space="preserve">Kliknięcie </t>
           </r>
           <r>
             <rPr>
@@ -3740,13 +3695,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Go to next page"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -3817,7 +3765,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>URL zawiera "</t>
+            <t xml:space="preserve">URL zawiera </t>
           </r>
           <r>
             <rPr>
@@ -3830,10 +3778,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>", info paginacji: "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">, info paginacji: </t>
           </r>
           <r>
             <rPr>
@@ -3848,7 +3795,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>", tabela pokazuje nowe wiersze</t>
+            <t>, tabela pokazuje nowe wiersze</t>
           </r>
         </is>
       </c>
@@ -3902,7 +3849,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>stan przycisku "</t>
+            <t xml:space="preserve">stan przycisku </t>
           </r>
           <r>
             <rPr>
@@ -3911,13 +3858,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Go to previous page"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -3964,7 +3904,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Przycisk "</t>
+            <t xml:space="preserve">Przycisk </t>
           </r>
           <r>
             <rPr>
@@ -3979,7 +3919,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" ma disabled=true, klik nie ma efektu</t>
+            <t xml:space="preserve"> ma disabled=true, klik nie ma efektu</t>
           </r>
         </is>
       </c>
@@ -4033,7 +3973,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>stan przycisku "</t>
+            <t xml:space="preserve">stan przycisku </t>
           </r>
           <r>
             <rPr>
@@ -4042,13 +3982,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Go to next page"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -4095,7 +4028,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Przycisk "</t>
+            <t xml:space="preserve">Przycisk </t>
           </r>
           <r>
             <rPr>
@@ -4108,10 +4041,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" ma disabled=true, info paginacji: "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> ma disabled=true, info paginacji: </t>
           </r>
           <r>
             <rPr>
@@ -4126,7 +4058,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>", tabela pokazuje 5 wierszy</t>
+            <t>, tabela pokazuje 5 wierszy</t>
           </r>
         </is>
       </c>
@@ -4930,7 +4862,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Wszystkie interaktywne elementy mają meaningful accessible names (WCAG 4.1.2), dynamiczne zmiany (nowy licznik, nowa lista, otwarcie modala) komunikowane (4.1.3), komunikat "</t>
+            <t xml:space="preserve">Wszystkie interaktywne elementy mają meaningful accessible names (WCAG 4.1.2), dynamiczne zmiany (nowy licznik, nowa lista, otwarcie modala) komunikowane (4.1.3), komunikat </t>
           </r>
           <r>
             <rPr>
@@ -4945,7 +4877,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" jest ogłaszany</t>
+            <t xml:space="preserve"> jest ogłaszany</t>
           </r>
         </is>
       </c>
@@ -5038,7 +4970,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Vistula → Znaleziono: 22, pierwszy wiersz: "</t>
+            <t xml:space="preserve">Vistula → Znaleziono: 22, pierwszy wiersz: </t>
           </r>
           <r>
             <rPr>
@@ -5047,13 +4979,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Akademia Finansów i Biznesu Vistula"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -5091,7 +5016,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Link "</t>
+            <t xml:space="preserve">Link </t>
           </r>
           <r>
             <rPr>
@@ -5104,10 +5029,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" ma target="</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> ma target=</t>
           </r>
           <r>
             <rPr>
@@ -5122,7 +5046,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">", href </t>
+            <t xml:space="preserve">, href </t>
           </r>
           <r>
             <rPr>
@@ -5176,7 +5100,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Link "</t>
+            <t xml:space="preserve">Link </t>
           </r>
           <r>
             <rPr>
@@ -5189,10 +5113,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" na stronie detali ma target="</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> na stronie detali ma target=</t>
           </r>
           <r>
             <rPr>
@@ -5205,10 +5128,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" + rel="</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> + rel=</t>
           </r>
           <r>
             <rPr>
@@ -5223,7 +5145,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" — bezpieczne otwarcie</t>
+            <t xml:space="preserve"> — bezpieczne otwarcie</t>
           </r>
         </is>
       </c>
@@ -5299,7 +5221,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Fraza "</t>
+            <t xml:space="preserve">Fraza </t>
           </r>
           <r>
             <rPr>
@@ -5312,10 +5234,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" → Znaleziono: 0, tabela "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> → Znaleziono: 0, tabela </t>
           </r>
           <r>
             <rPr>
@@ -5324,13 +5245,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Brak danych"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -5368,7 +5282,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>łódź=84, ŁÓDŹ=84 (wielkość liter ignorowana); "</t>
+            <t xml:space="preserve">łódź=84, ŁÓDŹ=84 (wielkość liter ignorowana); </t>
           </r>
           <r>
             <rPr>
@@ -5383,7 +5297,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" (z spacjami) = Vistula = 22 (spacje na krańcach przycięte); Filia; = 204 (średnik jako znak specjalny nie łamie wyszukiwania)</t>
+            <t xml:space="preserve"> (z spacjami) = Vistula = 22 (spacje na krańcach przycięte); Filia; = 204 (średnik jako znak specjalny nie łamie wyszukiwania)</t>
           </r>
         </is>
       </c>
@@ -5496,14 +5410,79 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0&amp;search=lodz</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> 2) Zapisz licznik (1) 3) Otwórz ?search=łódź (URL-encoded) 4) Porównaj (84)</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+2) W pole wyszukiwania wpisz frazę </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"lodz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (bez polskich znaków / bez ogonków)
+3) Poczekaj ~2–3s i zapisz licznik </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Znaleziono"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+4) Wyczyść pole (Cmd</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="FF0563C1"/>
+              <sz val="10"/>
+              <u val="single"/>
+            </rPr>
+            <t>/Ctrl</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">+A + Delete), wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"łódź"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (z polskimi znakami), poczekaj i zapisz licznik referencyjny (~84)
+5) Porównaj oba liczniki</t>
           </r>
         </is>
       </c>
@@ -5526,7 +5505,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>500-char query "</t>
+            <t xml:space="preserve">500-char query </t>
           </r>
           <r>
             <rPr>
@@ -5539,10 +5518,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" → 0 wyników, "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> → 0 wyników, </t>
           </r>
           <r>
             <rPr>
@@ -5555,10 +5533,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>", brak crashu. XSS payload "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">, brak crashu. XSS payload </t>
           </r>
           <r>
             <rPr>
@@ -5573,7 +5550,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" wyrenderowany jako tekst, brak execution, brak &lt;script&gt; w DOM. limit=abc normalizowany na 20, offset=-1 na -20 (dziwna normalizacja, ale bez crashu i stack trace)</t>
+            <t xml:space="preserve"> wyrenderowany jako tekst, brak execution, brak &lt;script&gt; w DOM. limit=abc normalizowany na 20, offset=-1 na -20 (dziwna normalizacja, ale bez crashu i stack trace)</t>
           </r>
         </is>
       </c>
@@ -5687,7 +5664,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Combobox Siedziba "</t>
+            <t xml:space="preserve">Combobox Siedziba </t>
           </r>
           <r>
             <rPr>
@@ -5702,7 +5679,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" → licznik 2605→350, URL &amp;cities=Warszawa</t>
+            <t xml:space="preserve"> → licznik 2605→350, URL &amp;cities=Warszawa</t>
           </r>
         </is>
       </c>
@@ -5778,7 +5755,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Klik ikony (i) obok "</t>
+            <t xml:space="preserve">Klik ikony (i) obok </t>
           </r>
           <r>
             <rPr>
@@ -5791,10 +5768,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" otworzył modal role=dialog z nagłówkiem "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> otworzył modal role=dialog z nagłówkiem </t>
           </r>
           <r>
             <rPr>
@@ -5807,10 +5783,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" i treścią: "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i treścią: </t>
           </r>
           <r>
             <rPr>
@@ -5819,13 +5794,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Instytucja certyfikująca (IC) – uprawniona instytucja…"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -5863,7 +5831,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>search=nieistniejaca_instytucja_xyz + roles=1 → Znaleziono: 0, "</t>
+            <t xml:space="preserve">search=nieistniejaca_instytucja_xyz + roles=1 → Znaleziono: 0, </t>
           </r>
           <r>
             <rPr>
@@ -5872,13 +5840,6 @@
               <sz val="10"/>
             </rPr>
             <t>"Brak danych"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"</t>
           </r>
         </is>
       </c>
@@ -5992,7 +5953,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Przycisk "</t>
+            <t xml:space="preserve">Przycisk </t>
           </r>
           <r>
             <rPr>
@@ -6005,10 +5966,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" nie jest disabled przy licznikiku 0. Pobrany plik ma 1 wiersz × 1 kolumnę, komórka = None (pusty XLSX bez nawet nagłówka "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> nie jest disabled przy licznikiku 0. Pobrany plik ma 1 wiersz × 1 kolumnę, komórka = None (pusty XLSX bez nawet nagłówka </t>
           </r>
           <r>
             <rPr>
@@ -6023,7 +5983,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>")</t>
+            <t>)</t>
           </r>
         </is>
       </c>
@@ -6053,7 +6013,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0&amp;search=nieistniejaca_xyz</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -6061,8 +6021,38 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Zaobserwuj Znaleziono: 0
-3) Kliknij </t>
+2) W pole wyszukiwania wpisz frazę </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"nieistniejaca_xyz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i poczekaj aż licznik pokaże </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Znaleziono: 0"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+3) Kliknij przycisk </t>
           </r>
           <r>
             <rPr>
@@ -6078,7 +6068,7 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-4) Otwórz plik: 1×1 arkusz, brak nagłówka, brak danych</t>
+4) Otwórz pobrany plik i sprawdź czy zawiera nagłówek kolumn</t>
           </r>
         </is>
       </c>
@@ -6101,7 +6091,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Klik Next na offset=0 → URL ?limit=20&amp;offset=20, info paginacji "</t>
+            <t xml:space="preserve">Klik Next na offset=0 → URL ?limit=20&amp;offset=20, info paginacji </t>
           </r>
           <r>
             <rPr>
@@ -6116,7 +6106,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>", tabela pokazała nowe wiersze</t>
+            <t>, tabela pokazała nowe wiersze</t>
           </r>
         </is>
       </c>
@@ -6154,7 +6144,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Na offset=0 przycisk "</t>
+            <t xml:space="preserve">Na offset=0 przycisk </t>
           </r>
           <r>
             <rPr>
@@ -6169,7 +6159,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>" ma disabled=true</t>
+            <t xml:space="preserve"> ma disabled=true</t>
           </r>
         </is>
       </c>
@@ -6207,7 +6197,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Na offset=2600 przycisk "</t>
+            <t xml:space="preserve">Na offset=2600 przycisk </t>
           </r>
           <r>
             <rPr>
@@ -6220,10 +6210,9 @@
           <r>
             <rPr>
               <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>" ma disabled=true, info paginacji "</t>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> ma disabled=true, info paginacji </t>
           </r>
           <r>
             <rPr>
@@ -6238,7 +6227,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>", tabela pokazała 5 wierszy</t>
+            <t>, tabela pokazała 5 wierszy</t>
           </r>
         </is>
       </c>
@@ -6504,4 +6493,883 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FFC000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="85" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>INST-BR-01 — Wyszukiwarka nie znajduje polskich nazw gdy fraza wpisana bez polskich znaków</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Metadane</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>INST-BR-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Tytuł</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Wyszukiwarka nie znajduje polskich nazw gdy fraza wpisana bez polskich znaków</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Priorytet</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>P2 · Wysoki</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Ważność</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Powiązany scenariusz testowy</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>INST-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Data zgłoszenia</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Środowisko</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="FF0563C1"/>
+              <sz val="10"/>
+              <u val="single"/>
+            </rPr>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Przeglądarka</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Chrome (latest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>System operacyjny</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>macOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Rozdzielczość</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>1440×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Reprodukcja</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="144" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Kroki reprodukcji</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">1) Otwórz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="FF0563C1"/>
+              <sz val="10"/>
+              <u val="single"/>
+            </rPr>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+2) W pole wyszukiwania wpisz frazę </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"lodz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (bez polskich znaków / bez ogonków)
+3) Poczekaj ~2–3s i zapisz licznik </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Znaleziono"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+4) Wyczyść pole (Cmd</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="FF0563C1"/>
+              <sz val="10"/>
+              <u val="single"/>
+            </rPr>
+            <t>/Ctrl</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">+A + Delete), wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"łódź"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (z polskimi znakami), poczekaj i zapisz licznik referencyjny (~84)
+5) Porównaj oba liczniki</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Oczekiwany rezultat</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">Licznik dla </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"lodz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> ≈ licznik dla </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"łódź"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (~84); backend normalizuje diakrytyki (unaccent / asciifolding) i znajduje nazwy z </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Łódź"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> niezależnie od tego czy user wpisał </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"lodz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> czy </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"łódź"</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Rzeczywisty rezultat</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"lodz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (bez ogonków) → Znaleziono: 1; </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"łódź"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> (z ogonkami) → Znaleziono: 84. Backend nie wykonuje asciifolding / unaccent — użytkownik piszący </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"lodz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> traci 83 wyniki, które faktycznie zawierają </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Łódź"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> w nazwie</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Screenshot</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>qa-runs/screenshots/INST-07.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Analiza wpływu</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="64" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">Użytkownicy piszący na klawiaturze angielskiej lub na klawiaturze mobilnej bez polskich znaków tracą 83 z 84 wyników zawierających </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Łódź"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> — nie znajdują szukanej instytucji, myślą że jej nie ma w bazie. Realne dla znaczącej części ruchu (&gt;60% traffic mobile w PL, klawiatura EN u wielu użytkowników desktop).</t>
+          </r>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A9:B9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00A6A6A6"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="85" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>INST-BR-02 — Pobieranie przy zerowych wynikach generuje pusty plik XLSX bez nagłówka</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Metadane</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>INST-BR-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Tytuł</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Pobieranie przy zerowych wynikach generuje pusty plik XLSX bez nagłówka</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Priorytet</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>P3 · Niski</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Ważność</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Powiązany scenariusz testowy</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>INST-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Data zgłoszenia</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Środowisko</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="FF0563C1"/>
+              <sz val="10"/>
+              <u val="single"/>
+            </rPr>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Przeglądarka</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Chrome (latest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>System operacyjny</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>macOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Rozdzielczość</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>1440×900</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Reprodukcja</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="112" customHeight="1">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Kroki reprodukcji</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">1) Otwórz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="FF0563C1"/>
+              <sz val="10"/>
+              <u val="single"/>
+            </rPr>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+2) W pole wyszukiwania wpisz frazę </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"nieistniejaca_xyz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i poczekaj aż licznik pokaże </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Znaleziono: 0"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+3) Kliknij przycisk </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Pobierz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">
+4) Otwórz pobrany plik i sprawdź czy zawiera nagłówek kolumn</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Oczekiwany rezultat</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">Przycisk </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Pobierz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> jest wyłączony LUB pobrany plik zawiera co najmniej nagłówek kolumn (nie tylko pusty arkusz)</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Rzeczywisty rezultat</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">Przycisk </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Pobierz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> nie jest disabled przy liczniku 0. Pobrany plik ma 1 wiersz × 1 kolumnę, komórka = None (pusty XLSX bez nawet nagłówka </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"#/ID/Nazwa"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t>)</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Screenshot</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>qa-runs/screenshots/INST-17.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Analiza wpływu</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">Użytkownik przy pustym wyniku wyszukiwania klika </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Pobierz"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i dostaje niezrozumiały pusty plik zamiast informacji zwrotnej. Myślący że plik jest uszkodzony lub że eksport nie zadziałał. Rzadko trafia w flow (typowo user widzi 0 wyników i już nie pobiera), ale gdy trafi — mylące.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A9:B9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
qa-runs: apply PL severity + env versions + embedded screenshots
Applied all new bug report polish to wyszukiwarka-instytucji run.

Bug tracker + MDs:
- Kolumna: Ważność -> Ważność/dotkliwość
- INST-BR-01: Medium -> Średnia
- INST-BR-02: Low -> Niska
- Przegladarka: Chrome (latest) -> Chrome 151 (z Playwright user-agent)
- System operacyjny: macOS -> macOS 15.7.4 (z sw_vers -productVersion)

Execution report:
- Waga column values: Medium/Low -> Średnia/Niska (spojnosc z bug tracker)

XLSX zregenerowany z:
- Załączniki section z embedded real screenshots (~500KB rozmiar pliku
  po dodaniu 2 PNG-i)
- Bidirectional hyperlinki miedzy Test cases i bug tabs
- Section title bars (Metadane/Środowisko/Reprodukcja/Analiza wpływu/Załączniki)
- Priorytet + Ważność/dotkliwość color-coded

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
+++ b/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,8 +61,21 @@
       <color rgb="001F3864"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -114,6 +127,16 @@
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4E4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -141,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -176,6 +199,9 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -197,8 +223,14 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -274,6 +306,66 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6191250" cy="12668250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6191250" cy="3867150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2032,7 +2124,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr">
         <is>
           <t>INST-BR-01</t>
         </is>
@@ -3493,7 +3585,7 @@
           <t>Pobieranie przy zerowych wynikach nie generuje pustego pliku bez nagłówka</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C18" s="13" t="inlineStr">
         <is>
           <t>P3 · Niski</t>
         </is>
@@ -3641,7 +3733,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I18" s="12" t="inlineStr">
         <is>
           <t>INST-BR-02</t>
         </is>
@@ -4580,7 +4672,7 @@
           </r>
         </is>
       </c>
-      <c r="H25" s="13" t="inlineStr">
+      <c r="H25" s="14" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
@@ -4724,7 +4816,7 @@
           </r>
         </is>
       </c>
-      <c r="H26" s="13" t="inlineStr">
+      <c r="H26" s="14" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
@@ -4881,7 +4973,7 @@
           </r>
         </is>
       </c>
-      <c r="H27" s="13" t="inlineStr">
+      <c r="H27" s="14" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
@@ -4898,6 +4990,10 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5384,9 +5480,9 @@
           </r>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>Średnia</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -5987,9 +6083,9 @@
           </r>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>Niska</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -6382,7 +6478,7 @@
           <t>INST-24</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
@@ -6420,7 +6516,7 @@
           <t>INST-25</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
@@ -6458,7 +6554,7 @@
           <t>INST-26</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
@@ -6510,21 +6606,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>INST-BR-01 — Wyszukiwarka nie znajduje polskich nazw gdy fraza wpisana bez polskich znaków</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Metadane</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
@@ -6536,7 +6632,7 @@
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Tytuł</t>
         </is>
@@ -6548,43 +6644,43 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Priorytet</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>P2 · Wysoki</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>Ważność</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Ważność/dotkliwość</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Średnia</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Powiązany scenariusz testowy</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>INST-07</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Data zgłoszenia</t>
         </is>
@@ -6596,14 +6692,14 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Środowisko</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -6623,31 +6719,31 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Przeglądarka</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Chrome (latest)</t>
+          <t>Chrome 151</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>System operacyjny</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>macOS</t>
+          <t>macOS 15.7.4</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Rozdzielczość</t>
         </is>
@@ -6659,14 +6755,14 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Reprodukcja</t>
         </is>
       </c>
     </row>
     <row r="15" ht="144" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Kroki reprodukcji</t>
         </is>
@@ -6765,12 +6861,12 @@
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Oczekiwany rezultat</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6851,12 +6947,12 @@
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Rzeczywisty rezultat</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6921,27 +7017,20 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
+    <row r="18" ht="24" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
         <is>
-          <t>Screenshot</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>qa-runs/screenshots/INST-07.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
-        <is>
           <t>Analiza wpływu</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="64" customHeight="1">
-      <c r="A20" s="19" t="inlineStr">
+    <row r="19" ht="80" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Wpływ na użytkownika</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6968,16 +7057,116 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Załączniki</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1"/>
+    <row r="22" ht="15" customHeight="1"/>
+    <row r="23" ht="15" customHeight="1"/>
+    <row r="24" ht="15" customHeight="1"/>
+    <row r="25" ht="15" customHeight="1"/>
+    <row r="26" ht="15" customHeight="1"/>
+    <row r="27" ht="15" customHeight="1"/>
+    <row r="28" ht="15" customHeight="1"/>
+    <row r="29" ht="15" customHeight="1"/>
+    <row r="30" ht="15" customHeight="1"/>
+    <row r="31" ht="15" customHeight="1"/>
+    <row r="32" ht="15" customHeight="1"/>
+    <row r="33" ht="15" customHeight="1"/>
+    <row r="34" ht="15" customHeight="1"/>
+    <row r="35" ht="15" customHeight="1"/>
+    <row r="36" ht="15" customHeight="1"/>
+    <row r="37" ht="15" customHeight="1"/>
+    <row r="38" ht="15" customHeight="1"/>
+    <row r="39" ht="15" customHeight="1"/>
+    <row r="40" ht="15" customHeight="1"/>
+    <row r="41" ht="15" customHeight="1"/>
+    <row r="42" ht="15" customHeight="1"/>
+    <row r="43" ht="15" customHeight="1"/>
+    <row r="44" ht="15" customHeight="1"/>
+    <row r="45" ht="15" customHeight="1"/>
+    <row r="46" ht="15" customHeight="1"/>
+    <row r="47" ht="15" customHeight="1"/>
+    <row r="48" ht="15" customHeight="1"/>
+    <row r="49" ht="15" customHeight="1"/>
+    <row r="50" ht="15" customHeight="1"/>
+    <row r="51" ht="15" customHeight="1"/>
+    <row r="52" ht="15" customHeight="1"/>
+    <row r="53" ht="15" customHeight="1"/>
+    <row r="54" ht="15" customHeight="1"/>
+    <row r="55" ht="15" customHeight="1"/>
+    <row r="56" ht="15" customHeight="1"/>
+    <row r="57" ht="15" customHeight="1"/>
+    <row r="58" ht="15" customHeight="1"/>
+    <row r="59" ht="15" customHeight="1"/>
+    <row r="60" ht="15" customHeight="1"/>
+    <row r="61" ht="15" customHeight="1"/>
+    <row r="62" ht="15" customHeight="1"/>
+    <row r="63" ht="15" customHeight="1"/>
+    <row r="64" ht="15" customHeight="1"/>
+    <row r="65" ht="15" customHeight="1"/>
+    <row r="66" ht="15" customHeight="1"/>
+    <row r="67" ht="15" customHeight="1"/>
+    <row r="68" ht="15" customHeight="1"/>
+    <row r="69" ht="15" customHeight="1"/>
+    <row r="70" ht="15" customHeight="1"/>
+    <row r="71" ht="15" customHeight="1"/>
+    <row r="72" ht="15" customHeight="1"/>
+    <row r="73" ht="15" customHeight="1"/>
+    <row r="74" ht="15" customHeight="1"/>
+    <row r="75" ht="15" customHeight="1"/>
+    <row r="76" ht="15" customHeight="1"/>
+    <row r="77" ht="15" customHeight="1"/>
+    <row r="78" ht="15" customHeight="1"/>
+    <row r="79" ht="15" customHeight="1"/>
+    <row r="80" ht="15" customHeight="1"/>
+    <row r="81" ht="15" customHeight="1"/>
+    <row r="82" ht="15" customHeight="1"/>
+    <row r="83" ht="15" customHeight="1"/>
+    <row r="84" ht="15" customHeight="1"/>
+    <row r="85" ht="15" customHeight="1"/>
+    <row r="86" ht="15" customHeight="1"/>
+    <row r="87" ht="15" customHeight="1"/>
+    <row r="88" ht="15" customHeight="1"/>
+    <row r="89" ht="15" customHeight="1"/>
+    <row r="90" ht="15" customHeight="1"/>
+    <row r="91" ht="15" customHeight="1"/>
+    <row r="92" ht="15" customHeight="1"/>
+    <row r="93" ht="15" customHeight="1"/>
+    <row r="94" ht="15" customHeight="1"/>
+    <row r="95" ht="15" customHeight="1"/>
+    <row r="96" ht="15" customHeight="1"/>
+    <row r="97" ht="15" customHeight="1"/>
+    <row r="98" ht="15" customHeight="1"/>
+    <row r="99" ht="15" customHeight="1"/>
+    <row r="100" ht="15" customHeight="1"/>
+    <row r="101" ht="15" customHeight="1"/>
+    <row r="102" ht="15" customHeight="1"/>
+    <row r="103" ht="15" customHeight="1"/>
+    <row r="104" ht="15" customHeight="1"/>
+    <row r="105" ht="15" customHeight="1"/>
+    <row r="106" ht="15" customHeight="1"/>
+    <row r="107" ht="15" customHeight="1"/>
+    <row r="108" ht="15" customHeight="1"/>
+    <row r="109" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A9:B9"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -6996,21 +7185,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>INST-BR-02 — Pobieranie przy zerowych wynikach generuje pusty plik XLSX bez nagłówka</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Metadane</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
@@ -7022,7 +7211,7 @@
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Tytuł</t>
         </is>
@@ -7034,43 +7223,43 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Priorytet</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>P3 · Niski</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>Ważność</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Ważność/dotkliwość</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Niska</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Powiązany scenariusz testowy</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>INST-17</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Data zgłoszenia</t>
         </is>
@@ -7082,14 +7271,14 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Środowisko</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -7109,31 +7298,31 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Przeglądarka</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Chrome (latest)</t>
+          <t>Chrome 151</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>System operacyjny</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>macOS</t>
+          <t>macOS 15.7.4</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Rozdzielczość</t>
         </is>
@@ -7145,14 +7334,14 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Reprodukcja</t>
         </is>
       </c>
     </row>
     <row r="15" ht="112" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Kroki reprodukcji</t>
         </is>
@@ -7234,12 +7423,12 @@
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Oczekiwany rezultat</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7267,12 +7456,12 @@
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Rzeczywisty rezultat</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7314,27 +7503,20 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
+    <row r="18" ht="24" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
         <is>
-          <t>Screenshot</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>qa-runs/screenshots/INST-17.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
-        <is>
           <t>Analiza wpływu</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1">
-      <c r="A20" s="19" t="inlineStr">
+    <row r="19" ht="64" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Wpływ na użytkownika</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7361,15 +7543,53 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Załączniki</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1"/>
+    <row r="22" ht="15" customHeight="1"/>
+    <row r="23" ht="15" customHeight="1"/>
+    <row r="24" ht="15" customHeight="1"/>
+    <row r="25" ht="15" customHeight="1"/>
+    <row r="26" ht="15" customHeight="1"/>
+    <row r="27" ht="15" customHeight="1"/>
+    <row r="28" ht="15" customHeight="1"/>
+    <row r="29" ht="15" customHeight="1"/>
+    <row r="30" ht="15" customHeight="1"/>
+    <row r="31" ht="15" customHeight="1"/>
+    <row r="32" ht="15" customHeight="1"/>
+    <row r="33" ht="15" customHeight="1"/>
+    <row r="34" ht="15" customHeight="1"/>
+    <row r="35" ht="15" customHeight="1"/>
+    <row r="36" ht="15" customHeight="1"/>
+    <row r="37" ht="15" customHeight="1"/>
+    <row r="38" ht="15" customHeight="1"/>
+    <row r="39" ht="15" customHeight="1"/>
+    <row r="40" ht="15" customHeight="1"/>
+    <row r="41" ht="15" customHeight="1"/>
+    <row r="42" ht="15" customHeight="1"/>
+    <row r="43" ht="15" customHeight="1"/>
+    <row r="44" ht="15" customHeight="1"/>
+    <row r="45" ht="15" customHeight="1"/>
+    <row r="46" ht="15" customHeight="1"/>
+    <row r="47" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A9:B9"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(/qa-case): bug tab visual polish — hide C+ columns + thick frame around A:B
Bug per-tab XLSX cleanup:
- Ukryj wszystkie kolumny poza A:B — jeden ColumnDimension range
  (min=3, max=16384=XFD) zamiast 16k obiektów, XML kompaktowy
- Thick dark blue border (#305496, medium weight) wokół całego content
  A:B — górna krawędź title bar, dolna krawędź ostatniego wiersza,
  boczne krawędzie lewa A + prawa B
- Bug tab wyglada teraz jak "karta" bez wystających pustych kolumn

Test cases + Execution report bez zmian (używają wielu kolumn).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
+++ b/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
@@ -138,7 +138,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -160,11 +160,95 @@
         <color rgb="00D0D0D0"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="00305496"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="00305496"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00305496"/>
+      </right>
+      <top style="medium">
+        <color rgb="00305496"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00305496"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00305496"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D0D0"/>
+      </left>
+      <right style="medium">
+        <color rgb="00305496"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00305496"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00305496"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00305496"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00305496"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00305496"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -214,23 +298,37 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6598,11 +6696,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="85" customWidth="1" min="2" max="2"/>
+    <col hidden="1" width="13" customWidth="1" min="3" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -6611,100 +6710,103 @@
           <t>INST-BR-01 — Wyszukiwarka nie znajduje polskich nazw gdy fraza wpisana bez polskich znaków</t>
         </is>
       </c>
+      <c r="B1" s="18" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Metadane</t>
         </is>
       </c>
+      <c r="B2" s="20" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>INST-BR-01</t>
         </is>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Tytuł</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Wyszukiwarka nie znajduje polskich nazw gdy fraza wpisana bez polskich znaków</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Priorytet</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>P2 · Wysoki</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Ważność/dotkliwość</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Średnia</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Powiązany scenariusz testowy</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>INST-07</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Data zgłoszenia</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Środowisko</t>
         </is>
       </c>
+      <c r="B9" s="20" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6719,55 +6821,56 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Przeglądarka</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>Chrome 151</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>System operacyjny</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>macOS 15.7.4</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Rozdzielczość</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>1440×900</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Reprodukcja</t>
         </is>
       </c>
+      <c r="B14" s="20" t="n"/>
     </row>
     <row r="15" ht="144" customHeight="1">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Kroki reprodukcji</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6861,12 +6964,12 @@
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Oczekiwany rezultat</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6947,12 +7050,12 @@
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Rzeczywisty rezultat</t>
         </is>
       </c>
-      <c r="B17" s="22" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7018,19 +7121,20 @@
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Analiza wpływu</t>
         </is>
       </c>
+      <c r="B18" s="20" t="n"/>
     </row>
     <row r="19" ht="80" customHeight="1">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Wpływ na użytkownika</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7058,101 +7162,369 @@
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Załączniki</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="15" customHeight="1"/>
-    <row r="22" ht="15" customHeight="1"/>
-    <row r="23" ht="15" customHeight="1"/>
-    <row r="24" ht="15" customHeight="1"/>
-    <row r="25" ht="15" customHeight="1"/>
-    <row r="26" ht="15" customHeight="1"/>
-    <row r="27" ht="15" customHeight="1"/>
-    <row r="28" ht="15" customHeight="1"/>
-    <row r="29" ht="15" customHeight="1"/>
-    <row r="30" ht="15" customHeight="1"/>
-    <row r="31" ht="15" customHeight="1"/>
-    <row r="32" ht="15" customHeight="1"/>
-    <row r="33" ht="15" customHeight="1"/>
-    <row r="34" ht="15" customHeight="1"/>
-    <row r="35" ht="15" customHeight="1"/>
-    <row r="36" ht="15" customHeight="1"/>
-    <row r="37" ht="15" customHeight="1"/>
-    <row r="38" ht="15" customHeight="1"/>
-    <row r="39" ht="15" customHeight="1"/>
-    <row r="40" ht="15" customHeight="1"/>
-    <row r="41" ht="15" customHeight="1"/>
-    <row r="42" ht="15" customHeight="1"/>
-    <row r="43" ht="15" customHeight="1"/>
-    <row r="44" ht="15" customHeight="1"/>
-    <row r="45" ht="15" customHeight="1"/>
-    <row r="46" ht="15" customHeight="1"/>
-    <row r="47" ht="15" customHeight="1"/>
-    <row r="48" ht="15" customHeight="1"/>
-    <row r="49" ht="15" customHeight="1"/>
-    <row r="50" ht="15" customHeight="1"/>
-    <row r="51" ht="15" customHeight="1"/>
-    <row r="52" ht="15" customHeight="1"/>
-    <row r="53" ht="15" customHeight="1"/>
-    <row r="54" ht="15" customHeight="1"/>
-    <row r="55" ht="15" customHeight="1"/>
-    <row r="56" ht="15" customHeight="1"/>
-    <row r="57" ht="15" customHeight="1"/>
-    <row r="58" ht="15" customHeight="1"/>
-    <row r="59" ht="15" customHeight="1"/>
-    <row r="60" ht="15" customHeight="1"/>
-    <row r="61" ht="15" customHeight="1"/>
-    <row r="62" ht="15" customHeight="1"/>
-    <row r="63" ht="15" customHeight="1"/>
-    <row r="64" ht="15" customHeight="1"/>
-    <row r="65" ht="15" customHeight="1"/>
-    <row r="66" ht="15" customHeight="1"/>
-    <row r="67" ht="15" customHeight="1"/>
-    <row r="68" ht="15" customHeight="1"/>
-    <row r="69" ht="15" customHeight="1"/>
-    <row r="70" ht="15" customHeight="1"/>
-    <row r="71" ht="15" customHeight="1"/>
-    <row r="72" ht="15" customHeight="1"/>
-    <row r="73" ht="15" customHeight="1"/>
-    <row r="74" ht="15" customHeight="1"/>
-    <row r="75" ht="15" customHeight="1"/>
-    <row r="76" ht="15" customHeight="1"/>
-    <row r="77" ht="15" customHeight="1"/>
-    <row r="78" ht="15" customHeight="1"/>
-    <row r="79" ht="15" customHeight="1"/>
-    <row r="80" ht="15" customHeight="1"/>
-    <row r="81" ht="15" customHeight="1"/>
-    <row r="82" ht="15" customHeight="1"/>
-    <row r="83" ht="15" customHeight="1"/>
-    <row r="84" ht="15" customHeight="1"/>
-    <row r="85" ht="15" customHeight="1"/>
-    <row r="86" ht="15" customHeight="1"/>
-    <row r="87" ht="15" customHeight="1"/>
-    <row r="88" ht="15" customHeight="1"/>
-    <row r="89" ht="15" customHeight="1"/>
-    <row r="90" ht="15" customHeight="1"/>
-    <row r="91" ht="15" customHeight="1"/>
-    <row r="92" ht="15" customHeight="1"/>
-    <row r="93" ht="15" customHeight="1"/>
-    <row r="94" ht="15" customHeight="1"/>
-    <row r="95" ht="15" customHeight="1"/>
-    <row r="96" ht="15" customHeight="1"/>
-    <row r="97" ht="15" customHeight="1"/>
-    <row r="98" ht="15" customHeight="1"/>
-    <row r="99" ht="15" customHeight="1"/>
-    <row r="100" ht="15" customHeight="1"/>
-    <row r="101" ht="15" customHeight="1"/>
-    <row r="102" ht="15" customHeight="1"/>
-    <row r="103" ht="15" customHeight="1"/>
-    <row r="104" ht="15" customHeight="1"/>
-    <row r="105" ht="15" customHeight="1"/>
-    <row r="106" ht="15" customHeight="1"/>
-    <row r="107" ht="15" customHeight="1"/>
-    <row r="108" ht="15" customHeight="1"/>
-    <row r="109" ht="15" customHeight="1"/>
+      <c r="B20" s="20" t="n"/>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="27" t="n"/>
+      <c r="B21" s="20" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="27" t="n"/>
+      <c r="B22" s="20" t="n"/>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="27" t="n"/>
+      <c r="B23" s="20" t="n"/>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="27" t="n"/>
+      <c r="B24" s="20" t="n"/>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="27" t="n"/>
+      <c r="B25" s="20" t="n"/>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" s="27" t="n"/>
+      <c r="B26" s="20" t="n"/>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="27" t="n"/>
+      <c r="B27" s="20" t="n"/>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="27" t="n"/>
+      <c r="B28" s="20" t="n"/>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" s="27" t="n"/>
+      <c r="B29" s="20" t="n"/>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="27" t="n"/>
+      <c r="B30" s="20" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" s="27" t="n"/>
+      <c r="B31" s="20" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="27" t="n"/>
+      <c r="B32" s="20" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" s="27" t="n"/>
+      <c r="B33" s="20" t="n"/>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="A34" s="27" t="n"/>
+      <c r="B34" s="20" t="n"/>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="A35" s="27" t="n"/>
+      <c r="B35" s="20" t="n"/>
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="A36" s="27" t="n"/>
+      <c r="B36" s="20" t="n"/>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="27" t="n"/>
+      <c r="B37" s="20" t="n"/>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="27" t="n"/>
+      <c r="B38" s="20" t="n"/>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="27" t="n"/>
+      <c r="B39" s="20" t="n"/>
+    </row>
+    <row r="40" ht="15" customHeight="1">
+      <c r="A40" s="27" t="n"/>
+      <c r="B40" s="20" t="n"/>
+    </row>
+    <row r="41" ht="15" customHeight="1">
+      <c r="A41" s="27" t="n"/>
+      <c r="B41" s="20" t="n"/>
+    </row>
+    <row r="42" ht="15" customHeight="1">
+      <c r="A42" s="27" t="n"/>
+      <c r="B42" s="20" t="n"/>
+    </row>
+    <row r="43" ht="15" customHeight="1">
+      <c r="A43" s="27" t="n"/>
+      <c r="B43" s="20" t="n"/>
+    </row>
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" s="27" t="n"/>
+      <c r="B44" s="20" t="n"/>
+    </row>
+    <row r="45" ht="15" customHeight="1">
+      <c r="A45" s="27" t="n"/>
+      <c r="B45" s="20" t="n"/>
+    </row>
+    <row r="46" ht="15" customHeight="1">
+      <c r="A46" s="27" t="n"/>
+      <c r="B46" s="20" t="n"/>
+    </row>
+    <row r="47" ht="15" customHeight="1">
+      <c r="A47" s="27" t="n"/>
+      <c r="B47" s="20" t="n"/>
+    </row>
+    <row r="48" ht="15" customHeight="1">
+      <c r="A48" s="27" t="n"/>
+      <c r="B48" s="20" t="n"/>
+    </row>
+    <row r="49" ht="15" customHeight="1">
+      <c r="A49" s="27" t="n"/>
+      <c r="B49" s="20" t="n"/>
+    </row>
+    <row r="50" ht="15" customHeight="1">
+      <c r="A50" s="27" t="n"/>
+      <c r="B50" s="20" t="n"/>
+    </row>
+    <row r="51" ht="15" customHeight="1">
+      <c r="A51" s="27" t="n"/>
+      <c r="B51" s="20" t="n"/>
+    </row>
+    <row r="52" ht="15" customHeight="1">
+      <c r="A52" s="27" t="n"/>
+      <c r="B52" s="20" t="n"/>
+    </row>
+    <row r="53" ht="15" customHeight="1">
+      <c r="A53" s="27" t="n"/>
+      <c r="B53" s="20" t="n"/>
+    </row>
+    <row r="54" ht="15" customHeight="1">
+      <c r="A54" s="27" t="n"/>
+      <c r="B54" s="20" t="n"/>
+    </row>
+    <row r="55" ht="15" customHeight="1">
+      <c r="A55" s="27" t="n"/>
+      <c r="B55" s="20" t="n"/>
+    </row>
+    <row r="56" ht="15" customHeight="1">
+      <c r="A56" s="27" t="n"/>
+      <c r="B56" s="20" t="n"/>
+    </row>
+    <row r="57" ht="15" customHeight="1">
+      <c r="A57" s="27" t="n"/>
+      <c r="B57" s="20" t="n"/>
+    </row>
+    <row r="58" ht="15" customHeight="1">
+      <c r="A58" s="27" t="n"/>
+      <c r="B58" s="20" t="n"/>
+    </row>
+    <row r="59" ht="15" customHeight="1">
+      <c r="A59" s="27" t="n"/>
+      <c r="B59" s="20" t="n"/>
+    </row>
+    <row r="60" ht="15" customHeight="1">
+      <c r="A60" s="27" t="n"/>
+      <c r="B60" s="20" t="n"/>
+    </row>
+    <row r="61" ht="15" customHeight="1">
+      <c r="A61" s="27" t="n"/>
+      <c r="B61" s="20" t="n"/>
+    </row>
+    <row r="62" ht="15" customHeight="1">
+      <c r="A62" s="27" t="n"/>
+      <c r="B62" s="20" t="n"/>
+    </row>
+    <row r="63" ht="15" customHeight="1">
+      <c r="A63" s="27" t="n"/>
+      <c r="B63" s="20" t="n"/>
+    </row>
+    <row r="64" ht="15" customHeight="1">
+      <c r="A64" s="27" t="n"/>
+      <c r="B64" s="20" t="n"/>
+    </row>
+    <row r="65" ht="15" customHeight="1">
+      <c r="A65" s="27" t="n"/>
+      <c r="B65" s="20" t="n"/>
+    </row>
+    <row r="66" ht="15" customHeight="1">
+      <c r="A66" s="27" t="n"/>
+      <c r="B66" s="20" t="n"/>
+    </row>
+    <row r="67" ht="15" customHeight="1">
+      <c r="A67" s="27" t="n"/>
+      <c r="B67" s="20" t="n"/>
+    </row>
+    <row r="68" ht="15" customHeight="1">
+      <c r="A68" s="27" t="n"/>
+      <c r="B68" s="20" t="n"/>
+    </row>
+    <row r="69" ht="15" customHeight="1">
+      <c r="A69" s="27" t="n"/>
+      <c r="B69" s="20" t="n"/>
+    </row>
+    <row r="70" ht="15" customHeight="1">
+      <c r="A70" s="27" t="n"/>
+      <c r="B70" s="20" t="n"/>
+    </row>
+    <row r="71" ht="15" customHeight="1">
+      <c r="A71" s="27" t="n"/>
+      <c r="B71" s="20" t="n"/>
+    </row>
+    <row r="72" ht="15" customHeight="1">
+      <c r="A72" s="27" t="n"/>
+      <c r="B72" s="20" t="n"/>
+    </row>
+    <row r="73" ht="15" customHeight="1">
+      <c r="A73" s="27" t="n"/>
+      <c r="B73" s="20" t="n"/>
+    </row>
+    <row r="74" ht="15" customHeight="1">
+      <c r="A74" s="27" t="n"/>
+      <c r="B74" s="20" t="n"/>
+    </row>
+    <row r="75" ht="15" customHeight="1">
+      <c r="A75" s="27" t="n"/>
+      <c r="B75" s="20" t="n"/>
+    </row>
+    <row r="76" ht="15" customHeight="1">
+      <c r="A76" s="27" t="n"/>
+      <c r="B76" s="20" t="n"/>
+    </row>
+    <row r="77" ht="15" customHeight="1">
+      <c r="A77" s="27" t="n"/>
+      <c r="B77" s="20" t="n"/>
+    </row>
+    <row r="78" ht="15" customHeight="1">
+      <c r="A78" s="27" t="n"/>
+      <c r="B78" s="20" t="n"/>
+    </row>
+    <row r="79" ht="15" customHeight="1">
+      <c r="A79" s="27" t="n"/>
+      <c r="B79" s="20" t="n"/>
+    </row>
+    <row r="80" ht="15" customHeight="1">
+      <c r="A80" s="27" t="n"/>
+      <c r="B80" s="20" t="n"/>
+    </row>
+    <row r="81" ht="15" customHeight="1">
+      <c r="A81" s="27" t="n"/>
+      <c r="B81" s="20" t="n"/>
+    </row>
+    <row r="82" ht="15" customHeight="1">
+      <c r="A82" s="27" t="n"/>
+      <c r="B82" s="20" t="n"/>
+    </row>
+    <row r="83" ht="15" customHeight="1">
+      <c r="A83" s="27" t="n"/>
+      <c r="B83" s="20" t="n"/>
+    </row>
+    <row r="84" ht="15" customHeight="1">
+      <c r="A84" s="27" t="n"/>
+      <c r="B84" s="20" t="n"/>
+    </row>
+    <row r="85" ht="15" customHeight="1">
+      <c r="A85" s="27" t="n"/>
+      <c r="B85" s="20" t="n"/>
+    </row>
+    <row r="86" ht="15" customHeight="1">
+      <c r="A86" s="27" t="n"/>
+      <c r="B86" s="20" t="n"/>
+    </row>
+    <row r="87" ht="15" customHeight="1">
+      <c r="A87" s="27" t="n"/>
+      <c r="B87" s="20" t="n"/>
+    </row>
+    <row r="88" ht="15" customHeight="1">
+      <c r="A88" s="27" t="n"/>
+      <c r="B88" s="20" t="n"/>
+    </row>
+    <row r="89" ht="15" customHeight="1">
+      <c r="A89" s="27" t="n"/>
+      <c r="B89" s="20" t="n"/>
+    </row>
+    <row r="90" ht="15" customHeight="1">
+      <c r="A90" s="27" t="n"/>
+      <c r="B90" s="20" t="n"/>
+    </row>
+    <row r="91" ht="15" customHeight="1">
+      <c r="A91" s="27" t="n"/>
+      <c r="B91" s="20" t="n"/>
+    </row>
+    <row r="92" ht="15" customHeight="1">
+      <c r="A92" s="27" t="n"/>
+      <c r="B92" s="20" t="n"/>
+    </row>
+    <row r="93" ht="15" customHeight="1">
+      <c r="A93" s="27" t="n"/>
+      <c r="B93" s="20" t="n"/>
+    </row>
+    <row r="94" ht="15" customHeight="1">
+      <c r="A94" s="27" t="n"/>
+      <c r="B94" s="20" t="n"/>
+    </row>
+    <row r="95" ht="15" customHeight="1">
+      <c r="A95" s="27" t="n"/>
+      <c r="B95" s="20" t="n"/>
+    </row>
+    <row r="96" ht="15" customHeight="1">
+      <c r="A96" s="27" t="n"/>
+      <c r="B96" s="20" t="n"/>
+    </row>
+    <row r="97" ht="15" customHeight="1">
+      <c r="A97" s="27" t="n"/>
+      <c r="B97" s="20" t="n"/>
+    </row>
+    <row r="98" ht="15" customHeight="1">
+      <c r="A98" s="27" t="n"/>
+      <c r="B98" s="20" t="n"/>
+    </row>
+    <row r="99" ht="15" customHeight="1">
+      <c r="A99" s="27" t="n"/>
+      <c r="B99" s="20" t="n"/>
+    </row>
+    <row r="100" ht="15" customHeight="1">
+      <c r="A100" s="27" t="n"/>
+      <c r="B100" s="20" t="n"/>
+    </row>
+    <row r="101" ht="15" customHeight="1">
+      <c r="A101" s="27" t="n"/>
+      <c r="B101" s="20" t="n"/>
+    </row>
+    <row r="102" ht="15" customHeight="1">
+      <c r="A102" s="27" t="n"/>
+      <c r="B102" s="20" t="n"/>
+    </row>
+    <row r="103" ht="15" customHeight="1">
+      <c r="A103" s="27" t="n"/>
+      <c r="B103" s="20" t="n"/>
+    </row>
+    <row r="104" ht="15" customHeight="1">
+      <c r="A104" s="27" t="n"/>
+      <c r="B104" s="20" t="n"/>
+    </row>
+    <row r="105" ht="15" customHeight="1">
+      <c r="A105" s="27" t="n"/>
+      <c r="B105" s="20" t="n"/>
+    </row>
+    <row r="106" ht="15" customHeight="1">
+      <c r="A106" s="27" t="n"/>
+      <c r="B106" s="20" t="n"/>
+    </row>
+    <row r="107" ht="15" customHeight="1">
+      <c r="A107" s="27" t="n"/>
+      <c r="B107" s="20" t="n"/>
+    </row>
+    <row r="108" ht="15" customHeight="1">
+      <c r="A108" s="27" t="n"/>
+      <c r="B108" s="20" t="n"/>
+    </row>
+    <row r="109" ht="15" customHeight="1">
+      <c r="A109" s="28" t="n"/>
+      <c r="B109" s="29" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A20:B20"/>
@@ -7177,11 +7549,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="85" customWidth="1" min="2" max="2"/>
+    <col hidden="1" width="13" customWidth="1" min="3" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -7190,100 +7563,103 @@
           <t>INST-BR-02 — Pobieranie przy zerowych wynikach generuje pusty plik XLSX bez nagłówka</t>
         </is>
       </c>
+      <c r="B1" s="18" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Metadane</t>
         </is>
       </c>
+      <c r="B2" s="20" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>INST-BR-02</t>
         </is>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Tytuł</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Pobieranie przy zerowych wynikach generuje pusty plik XLSX bez nagłówka</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Priorytet</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>P3 · Niski</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Ważność/dotkliwość</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>Niska</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Powiązany scenariusz testowy</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>INST-17</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Data zgłoszenia</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Środowisko</t>
         </is>
       </c>
+      <c r="B9" s="20" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7298,55 +7674,56 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Przeglądarka</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>Chrome 151</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>System operacyjny</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>macOS 15.7.4</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Rozdzielczość</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>1440×900</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Reprodukcja</t>
         </is>
       </c>
+      <c r="B14" s="20" t="n"/>
     </row>
     <row r="15" ht="112" customHeight="1">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Kroki reprodukcji</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7423,12 +7800,12 @@
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Oczekiwany rezultat</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7456,12 +7833,12 @@
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Rzeczywisty rezultat</t>
         </is>
       </c>
-      <c r="B17" s="22" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7504,19 +7881,20 @@
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Analiza wpływu</t>
         </is>
       </c>
+      <c r="B18" s="20" t="n"/>
     </row>
     <row r="19" ht="64" customHeight="1">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Wpływ na użytkownika</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7544,39 +7922,121 @@
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Załączniki</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="15" customHeight="1"/>
-    <row r="22" ht="15" customHeight="1"/>
-    <row r="23" ht="15" customHeight="1"/>
-    <row r="24" ht="15" customHeight="1"/>
-    <row r="25" ht="15" customHeight="1"/>
-    <row r="26" ht="15" customHeight="1"/>
-    <row r="27" ht="15" customHeight="1"/>
-    <row r="28" ht="15" customHeight="1"/>
-    <row r="29" ht="15" customHeight="1"/>
-    <row r="30" ht="15" customHeight="1"/>
-    <row r="31" ht="15" customHeight="1"/>
-    <row r="32" ht="15" customHeight="1"/>
-    <row r="33" ht="15" customHeight="1"/>
-    <row r="34" ht="15" customHeight="1"/>
-    <row r="35" ht="15" customHeight="1"/>
-    <row r="36" ht="15" customHeight="1"/>
-    <row r="37" ht="15" customHeight="1"/>
-    <row r="38" ht="15" customHeight="1"/>
-    <row r="39" ht="15" customHeight="1"/>
-    <row r="40" ht="15" customHeight="1"/>
-    <row r="41" ht="15" customHeight="1"/>
-    <row r="42" ht="15" customHeight="1"/>
-    <row r="43" ht="15" customHeight="1"/>
-    <row r="44" ht="15" customHeight="1"/>
-    <row r="45" ht="15" customHeight="1"/>
-    <row r="46" ht="15" customHeight="1"/>
-    <row r="47" ht="15" customHeight="1"/>
+      <c r="B20" s="20" t="n"/>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="27" t="n"/>
+      <c r="B21" s="20" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="27" t="n"/>
+      <c r="B22" s="20" t="n"/>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="27" t="n"/>
+      <c r="B23" s="20" t="n"/>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="27" t="n"/>
+      <c r="B24" s="20" t="n"/>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="27" t="n"/>
+      <c r="B25" s="20" t="n"/>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" s="27" t="n"/>
+      <c r="B26" s="20" t="n"/>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="A27" s="27" t="n"/>
+      <c r="B27" s="20" t="n"/>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="27" t="n"/>
+      <c r="B28" s="20" t="n"/>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" s="27" t="n"/>
+      <c r="B29" s="20" t="n"/>
+    </row>
+    <row r="30" ht="15" customHeight="1">
+      <c r="A30" s="27" t="n"/>
+      <c r="B30" s="20" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" s="27" t="n"/>
+      <c r="B31" s="20" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="27" t="n"/>
+      <c r="B32" s="20" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" s="27" t="n"/>
+      <c r="B33" s="20" t="n"/>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="A34" s="27" t="n"/>
+      <c r="B34" s="20" t="n"/>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="A35" s="27" t="n"/>
+      <c r="B35" s="20" t="n"/>
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="A36" s="27" t="n"/>
+      <c r="B36" s="20" t="n"/>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="27" t="n"/>
+      <c r="B37" s="20" t="n"/>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="27" t="n"/>
+      <c r="B38" s="20" t="n"/>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="27" t="n"/>
+      <c r="B39" s="20" t="n"/>
+    </row>
+    <row r="40" ht="15" customHeight="1">
+      <c r="A40" s="27" t="n"/>
+      <c r="B40" s="20" t="n"/>
+    </row>
+    <row r="41" ht="15" customHeight="1">
+      <c r="A41" s="27" t="n"/>
+      <c r="B41" s="20" t="n"/>
+    </row>
+    <row r="42" ht="15" customHeight="1">
+      <c r="A42" s="27" t="n"/>
+      <c r="B42" s="20" t="n"/>
+    </row>
+    <row r="43" ht="15" customHeight="1">
+      <c r="A43" s="27" t="n"/>
+      <c r="B43" s="20" t="n"/>
+    </row>
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" s="27" t="n"/>
+      <c r="B44" s="20" t="n"/>
+    </row>
+    <row r="45" ht="15" customHeight="1">
+      <c r="A45" s="27" t="n"/>
+      <c r="B45" s="20" t="n"/>
+    </row>
+    <row r="46" ht="15" customHeight="1">
+      <c r="A46" s="27" t="n"/>
+      <c r="B46" s="20" t="n"/>
+    </row>
+    <row r="47" ht="15" customHeight="1">
+      <c r="A47" s="28" t="n"/>
+      <c r="B47" s="29" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A20:B20"/>

</xml_diff>

<commit_message>
feat(/qa-case): usun niebieska ramke + wydziel Rezultat jako osobna sekcja
Wizualne uproszczenia bug reportu:
- Usuniete thick dark blue frame wokol A:B (user nie chcial ramki mimo
  ukrytych C+ columns). Zostaje tylko cienki szary border miedzy cellkami.
- Sekcja "Reprodukcja" podzielona:
  - Reprodukcja (1 pole: Kroki reprodukcji)
  - Rezultat (2 pola: Oczekiwany rezultat zielony + Rzeczywisty rezultat
    czerwony) — nowa belka w tym samym stylu co inne sekcje

Nowa struktura per-bug (6 sekcji):
Metadane -> Środowisko -> Reprodukcja -> Rezultat -> Analiza wpływu -> Załączniki

Doc update: bug-report.md odzwierciedla nową strukturę + kolorowe tła
w sekcji Rezultat.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
+++ b/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
@@ -138,7 +138,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -160,95 +160,11 @@
         <color rgb="00D0D0D0"/>
       </bottom>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="00305496"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="00305496"/>
-      </top>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="00305496"/>
-      </right>
-      <top style="medium">
-        <color rgb="00305496"/>
-      </top>
-      <bottom/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="00305496"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D0D0D0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D0D0D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D0D0D0"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="00305496"/>
-      </right>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D0D0D0"/>
-      </left>
-      <right style="medium">
-        <color rgb="00305496"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D0D0D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D0D0D0"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="00305496"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="00305496"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="00305496"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="00305496"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="00305496"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -298,37 +214,23 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -412,7 +314,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6191250" cy="12668250"/>
@@ -442,7 +344,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>20</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6191250" cy="3867150"/>
@@ -6696,7 +6598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B109"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6710,103 +6612,100 @@
           <t>INST-BR-01 — Wyszukiwarka nie znajduje polskich nazw gdy fraza wpisana bez polskich znaków</t>
         </is>
       </c>
-      <c r="B1" s="18" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Metadane</t>
         </is>
       </c>
-      <c r="B2" s="20" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B3" s="22" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>INST-BR-01</t>
         </is>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Tytuł</t>
         </is>
       </c>
-      <c r="B4" s="22" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Wyszukiwarka nie znajduje polskich nazw gdy fraza wpisana bez polskich znaków</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Priorytet</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>P2 · Wysoki</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Ważność/dotkliwość</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Średnia</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Powiązany scenariusz testowy</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>INST-07</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Data zgłoszenia</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Środowisko</t>
         </is>
       </c>
-      <c r="B9" s="20" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6821,56 +6720,55 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Przeglądarka</t>
         </is>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Chrome 151</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>System operacyjny</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>macOS 15.7.4</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Rozdzielczość</t>
         </is>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>1440×900</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Reprodukcja</t>
         </is>
       </c>
-      <c r="B14" s="20" t="n"/>
     </row>
     <row r="15" ht="144" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Kroki reprodukcji</t>
         </is>
       </c>
-      <c r="B15" s="22" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6963,13 +6861,20 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Rezultat</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Oczekiwany rezultat</t>
         </is>
       </c>
-      <c r="B16" s="25" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7049,13 +6954,13 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Rzeczywisty rezultat</t>
         </is>
       </c>
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7120,21 +7025,20 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="19" t="inlineStr">
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Analiza wpływu</t>
         </is>
       </c>
-      <c r="B18" s="20" t="n"/>
-    </row>
-    <row r="19" ht="80" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
+    </row>
+    <row r="20" ht="80" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Wpływ na użytkownika</t>
         </is>
       </c>
-      <c r="B19" s="22" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7161,377 +7065,110 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="19" t="inlineStr">
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>Załączniki</t>
         </is>
       </c>
-      <c r="B20" s="20" t="n"/>
-    </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="27" t="n"/>
-      <c r="B21" s="20" t="n"/>
-    </row>
-    <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="27" t="n"/>
-      <c r="B22" s="20" t="n"/>
-    </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="27" t="n"/>
-      <c r="B23" s="20" t="n"/>
-    </row>
-    <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="27" t="n"/>
-      <c r="B24" s="20" t="n"/>
-    </row>
-    <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="27" t="n"/>
-      <c r="B25" s="20" t="n"/>
-    </row>
-    <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="27" t="n"/>
-      <c r="B26" s="20" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="27" t="n"/>
-      <c r="B27" s="20" t="n"/>
-    </row>
-    <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="27" t="n"/>
-      <c r="B28" s="20" t="n"/>
-    </row>
-    <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="27" t="n"/>
-      <c r="B29" s="20" t="n"/>
-    </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="27" t="n"/>
-      <c r="B30" s="20" t="n"/>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="27" t="n"/>
-      <c r="B31" s="20" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="27" t="n"/>
-      <c r="B32" s="20" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="27" t="n"/>
-      <c r="B33" s="20" t="n"/>
-    </row>
-    <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="27" t="n"/>
-      <c r="B34" s="20" t="n"/>
-    </row>
-    <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="27" t="n"/>
-      <c r="B35" s="20" t="n"/>
-    </row>
-    <row r="36" ht="15" customHeight="1">
-      <c r="A36" s="27" t="n"/>
-      <c r="B36" s="20" t="n"/>
-    </row>
-    <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="27" t="n"/>
-      <c r="B37" s="20" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="27" t="n"/>
-      <c r="B38" s="20" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="27" t="n"/>
-      <c r="B39" s="20" t="n"/>
-    </row>
-    <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="27" t="n"/>
-      <c r="B40" s="20" t="n"/>
-    </row>
-    <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="27" t="n"/>
-      <c r="B41" s="20" t="n"/>
-    </row>
-    <row r="42" ht="15" customHeight="1">
-      <c r="A42" s="27" t="n"/>
-      <c r="B42" s="20" t="n"/>
-    </row>
-    <row r="43" ht="15" customHeight="1">
-      <c r="A43" s="27" t="n"/>
-      <c r="B43" s="20" t="n"/>
-    </row>
-    <row r="44" ht="15" customHeight="1">
-      <c r="A44" s="27" t="n"/>
-      <c r="B44" s="20" t="n"/>
-    </row>
-    <row r="45" ht="15" customHeight="1">
-      <c r="A45" s="27" t="n"/>
-      <c r="B45" s="20" t="n"/>
-    </row>
-    <row r="46" ht="15" customHeight="1">
-      <c r="A46" s="27" t="n"/>
-      <c r="B46" s="20" t="n"/>
-    </row>
-    <row r="47" ht="15" customHeight="1">
-      <c r="A47" s="27" t="n"/>
-      <c r="B47" s="20" t="n"/>
-    </row>
-    <row r="48" ht="15" customHeight="1">
-      <c r="A48" s="27" t="n"/>
-      <c r="B48" s="20" t="n"/>
-    </row>
-    <row r="49" ht="15" customHeight="1">
-      <c r="A49" s="27" t="n"/>
-      <c r="B49" s="20" t="n"/>
-    </row>
-    <row r="50" ht="15" customHeight="1">
-      <c r="A50" s="27" t="n"/>
-      <c r="B50" s="20" t="n"/>
-    </row>
-    <row r="51" ht="15" customHeight="1">
-      <c r="A51" s="27" t="n"/>
-      <c r="B51" s="20" t="n"/>
-    </row>
-    <row r="52" ht="15" customHeight="1">
-      <c r="A52" s="27" t="n"/>
-      <c r="B52" s="20" t="n"/>
-    </row>
-    <row r="53" ht="15" customHeight="1">
-      <c r="A53" s="27" t="n"/>
-      <c r="B53" s="20" t="n"/>
-    </row>
-    <row r="54" ht="15" customHeight="1">
-      <c r="A54" s="27" t="n"/>
-      <c r="B54" s="20" t="n"/>
-    </row>
-    <row r="55" ht="15" customHeight="1">
-      <c r="A55" s="27" t="n"/>
-      <c r="B55" s="20" t="n"/>
-    </row>
-    <row r="56" ht="15" customHeight="1">
-      <c r="A56" s="27" t="n"/>
-      <c r="B56" s="20" t="n"/>
-    </row>
-    <row r="57" ht="15" customHeight="1">
-      <c r="A57" s="27" t="n"/>
-      <c r="B57" s="20" t="n"/>
-    </row>
-    <row r="58" ht="15" customHeight="1">
-      <c r="A58" s="27" t="n"/>
-      <c r="B58" s="20" t="n"/>
-    </row>
-    <row r="59" ht="15" customHeight="1">
-      <c r="A59" s="27" t="n"/>
-      <c r="B59" s="20" t="n"/>
-    </row>
-    <row r="60" ht="15" customHeight="1">
-      <c r="A60" s="27" t="n"/>
-      <c r="B60" s="20" t="n"/>
-    </row>
-    <row r="61" ht="15" customHeight="1">
-      <c r="A61" s="27" t="n"/>
-      <c r="B61" s="20" t="n"/>
-    </row>
-    <row r="62" ht="15" customHeight="1">
-      <c r="A62" s="27" t="n"/>
-      <c r="B62" s="20" t="n"/>
-    </row>
-    <row r="63" ht="15" customHeight="1">
-      <c r="A63" s="27" t="n"/>
-      <c r="B63" s="20" t="n"/>
-    </row>
-    <row r="64" ht="15" customHeight="1">
-      <c r="A64" s="27" t="n"/>
-      <c r="B64" s="20" t="n"/>
-    </row>
-    <row r="65" ht="15" customHeight="1">
-      <c r="A65" s="27" t="n"/>
-      <c r="B65" s="20" t="n"/>
-    </row>
-    <row r="66" ht="15" customHeight="1">
-      <c r="A66" s="27" t="n"/>
-      <c r="B66" s="20" t="n"/>
-    </row>
-    <row r="67" ht="15" customHeight="1">
-      <c r="A67" s="27" t="n"/>
-      <c r="B67" s="20" t="n"/>
-    </row>
-    <row r="68" ht="15" customHeight="1">
-      <c r="A68" s="27" t="n"/>
-      <c r="B68" s="20" t="n"/>
-    </row>
-    <row r="69" ht="15" customHeight="1">
-      <c r="A69" s="27" t="n"/>
-      <c r="B69" s="20" t="n"/>
-    </row>
-    <row r="70" ht="15" customHeight="1">
-      <c r="A70" s="27" t="n"/>
-      <c r="B70" s="20" t="n"/>
-    </row>
-    <row r="71" ht="15" customHeight="1">
-      <c r="A71" s="27" t="n"/>
-      <c r="B71" s="20" t="n"/>
-    </row>
-    <row r="72" ht="15" customHeight="1">
-      <c r="A72" s="27" t="n"/>
-      <c r="B72" s="20" t="n"/>
-    </row>
-    <row r="73" ht="15" customHeight="1">
-      <c r="A73" s="27" t="n"/>
-      <c r="B73" s="20" t="n"/>
-    </row>
-    <row r="74" ht="15" customHeight="1">
-      <c r="A74" s="27" t="n"/>
-      <c r="B74" s="20" t="n"/>
-    </row>
-    <row r="75" ht="15" customHeight="1">
-      <c r="A75" s="27" t="n"/>
-      <c r="B75" s="20" t="n"/>
-    </row>
-    <row r="76" ht="15" customHeight="1">
-      <c r="A76" s="27" t="n"/>
-      <c r="B76" s="20" t="n"/>
-    </row>
-    <row r="77" ht="15" customHeight="1">
-      <c r="A77" s="27" t="n"/>
-      <c r="B77" s="20" t="n"/>
-    </row>
-    <row r="78" ht="15" customHeight="1">
-      <c r="A78" s="27" t="n"/>
-      <c r="B78" s="20" t="n"/>
-    </row>
-    <row r="79" ht="15" customHeight="1">
-      <c r="A79" s="27" t="n"/>
-      <c r="B79" s="20" t="n"/>
-    </row>
-    <row r="80" ht="15" customHeight="1">
-      <c r="A80" s="27" t="n"/>
-      <c r="B80" s="20" t="n"/>
-    </row>
-    <row r="81" ht="15" customHeight="1">
-      <c r="A81" s="27" t="n"/>
-      <c r="B81" s="20" t="n"/>
-    </row>
-    <row r="82" ht="15" customHeight="1">
-      <c r="A82" s="27" t="n"/>
-      <c r="B82" s="20" t="n"/>
-    </row>
-    <row r="83" ht="15" customHeight="1">
-      <c r="A83" s="27" t="n"/>
-      <c r="B83" s="20" t="n"/>
-    </row>
-    <row r="84" ht="15" customHeight="1">
-      <c r="A84" s="27" t="n"/>
-      <c r="B84" s="20" t="n"/>
-    </row>
-    <row r="85" ht="15" customHeight="1">
-      <c r="A85" s="27" t="n"/>
-      <c r="B85" s="20" t="n"/>
-    </row>
-    <row r="86" ht="15" customHeight="1">
-      <c r="A86" s="27" t="n"/>
-      <c r="B86" s="20" t="n"/>
-    </row>
-    <row r="87" ht="15" customHeight="1">
-      <c r="A87" s="27" t="n"/>
-      <c r="B87" s="20" t="n"/>
-    </row>
-    <row r="88" ht="15" customHeight="1">
-      <c r="A88" s="27" t="n"/>
-      <c r="B88" s="20" t="n"/>
-    </row>
-    <row r="89" ht="15" customHeight="1">
-      <c r="A89" s="27" t="n"/>
-      <c r="B89" s="20" t="n"/>
-    </row>
-    <row r="90" ht="15" customHeight="1">
-      <c r="A90" s="27" t="n"/>
-      <c r="B90" s="20" t="n"/>
-    </row>
-    <row r="91" ht="15" customHeight="1">
-      <c r="A91" s="27" t="n"/>
-      <c r="B91" s="20" t="n"/>
-    </row>
-    <row r="92" ht="15" customHeight="1">
-      <c r="A92" s="27" t="n"/>
-      <c r="B92" s="20" t="n"/>
-    </row>
-    <row r="93" ht="15" customHeight="1">
-      <c r="A93" s="27" t="n"/>
-      <c r="B93" s="20" t="n"/>
-    </row>
-    <row r="94" ht="15" customHeight="1">
-      <c r="A94" s="27" t="n"/>
-      <c r="B94" s="20" t="n"/>
-    </row>
-    <row r="95" ht="15" customHeight="1">
-      <c r="A95" s="27" t="n"/>
-      <c r="B95" s="20" t="n"/>
-    </row>
-    <row r="96" ht="15" customHeight="1">
-      <c r="A96" s="27" t="n"/>
-      <c r="B96" s="20" t="n"/>
-    </row>
-    <row r="97" ht="15" customHeight="1">
-      <c r="A97" s="27" t="n"/>
-      <c r="B97" s="20" t="n"/>
-    </row>
-    <row r="98" ht="15" customHeight="1">
-      <c r="A98" s="27" t="n"/>
-      <c r="B98" s="20" t="n"/>
-    </row>
-    <row r="99" ht="15" customHeight="1">
-      <c r="A99" s="27" t="n"/>
-      <c r="B99" s="20" t="n"/>
-    </row>
-    <row r="100" ht="15" customHeight="1">
-      <c r="A100" s="27" t="n"/>
-      <c r="B100" s="20" t="n"/>
-    </row>
-    <row r="101" ht="15" customHeight="1">
-      <c r="A101" s="27" t="n"/>
-      <c r="B101" s="20" t="n"/>
-    </row>
-    <row r="102" ht="15" customHeight="1">
-      <c r="A102" s="27" t="n"/>
-      <c r="B102" s="20" t="n"/>
-    </row>
-    <row r="103" ht="15" customHeight="1">
-      <c r="A103" s="27" t="n"/>
-      <c r="B103" s="20" t="n"/>
-    </row>
-    <row r="104" ht="15" customHeight="1">
-      <c r="A104" s="27" t="n"/>
-      <c r="B104" s="20" t="n"/>
-    </row>
-    <row r="105" ht="15" customHeight="1">
-      <c r="A105" s="27" t="n"/>
-      <c r="B105" s="20" t="n"/>
-    </row>
-    <row r="106" ht="15" customHeight="1">
-      <c r="A106" s="27" t="n"/>
-      <c r="B106" s="20" t="n"/>
-    </row>
-    <row r="107" ht="15" customHeight="1">
-      <c r="A107" s="27" t="n"/>
-      <c r="B107" s="20" t="n"/>
-    </row>
-    <row r="108" ht="15" customHeight="1">
-      <c r="A108" s="27" t="n"/>
-      <c r="B108" s="20" t="n"/>
-    </row>
-    <row r="109" ht="15" customHeight="1">
-      <c r="A109" s="28" t="n"/>
-      <c r="B109" s="29" t="n"/>
-    </row>
+    </row>
+    <row r="22" ht="15" customHeight="1"/>
+    <row r="23" ht="15" customHeight="1"/>
+    <row r="24" ht="15" customHeight="1"/>
+    <row r="25" ht="15" customHeight="1"/>
+    <row r="26" ht="15" customHeight="1"/>
+    <row r="27" ht="15" customHeight="1"/>
+    <row r="28" ht="15" customHeight="1"/>
+    <row r="29" ht="15" customHeight="1"/>
+    <row r="30" ht="15" customHeight="1"/>
+    <row r="31" ht="15" customHeight="1"/>
+    <row r="32" ht="15" customHeight="1"/>
+    <row r="33" ht="15" customHeight="1"/>
+    <row r="34" ht="15" customHeight="1"/>
+    <row r="35" ht="15" customHeight="1"/>
+    <row r="36" ht="15" customHeight="1"/>
+    <row r="37" ht="15" customHeight="1"/>
+    <row r="38" ht="15" customHeight="1"/>
+    <row r="39" ht="15" customHeight="1"/>
+    <row r="40" ht="15" customHeight="1"/>
+    <row r="41" ht="15" customHeight="1"/>
+    <row r="42" ht="15" customHeight="1"/>
+    <row r="43" ht="15" customHeight="1"/>
+    <row r="44" ht="15" customHeight="1"/>
+    <row r="45" ht="15" customHeight="1"/>
+    <row r="46" ht="15" customHeight="1"/>
+    <row r="47" ht="15" customHeight="1"/>
+    <row r="48" ht="15" customHeight="1"/>
+    <row r="49" ht="15" customHeight="1"/>
+    <row r="50" ht="15" customHeight="1"/>
+    <row r="51" ht="15" customHeight="1"/>
+    <row r="52" ht="15" customHeight="1"/>
+    <row r="53" ht="15" customHeight="1"/>
+    <row r="54" ht="15" customHeight="1"/>
+    <row r="55" ht="15" customHeight="1"/>
+    <row r="56" ht="15" customHeight="1"/>
+    <row r="57" ht="15" customHeight="1"/>
+    <row r="58" ht="15" customHeight="1"/>
+    <row r="59" ht="15" customHeight="1"/>
+    <row r="60" ht="15" customHeight="1"/>
+    <row r="61" ht="15" customHeight="1"/>
+    <row r="62" ht="15" customHeight="1"/>
+    <row r="63" ht="15" customHeight="1"/>
+    <row r="64" ht="15" customHeight="1"/>
+    <row r="65" ht="15" customHeight="1"/>
+    <row r="66" ht="15" customHeight="1"/>
+    <row r="67" ht="15" customHeight="1"/>
+    <row r="68" ht="15" customHeight="1"/>
+    <row r="69" ht="15" customHeight="1"/>
+    <row r="70" ht="15" customHeight="1"/>
+    <row r="71" ht="15" customHeight="1"/>
+    <row r="72" ht="15" customHeight="1"/>
+    <row r="73" ht="15" customHeight="1"/>
+    <row r="74" ht="15" customHeight="1"/>
+    <row r="75" ht="15" customHeight="1"/>
+    <row r="76" ht="15" customHeight="1"/>
+    <row r="77" ht="15" customHeight="1"/>
+    <row r="78" ht="15" customHeight="1"/>
+    <row r="79" ht="15" customHeight="1"/>
+    <row r="80" ht="15" customHeight="1"/>
+    <row r="81" ht="15" customHeight="1"/>
+    <row r="82" ht="15" customHeight="1"/>
+    <row r="83" ht="15" customHeight="1"/>
+    <row r="84" ht="15" customHeight="1"/>
+    <row r="85" ht="15" customHeight="1"/>
+    <row r="86" ht="15" customHeight="1"/>
+    <row r="87" ht="15" customHeight="1"/>
+    <row r="88" ht="15" customHeight="1"/>
+    <row r="89" ht="15" customHeight="1"/>
+    <row r="90" ht="15" customHeight="1"/>
+    <row r="91" ht="15" customHeight="1"/>
+    <row r="92" ht="15" customHeight="1"/>
+    <row r="93" ht="15" customHeight="1"/>
+    <row r="94" ht="15" customHeight="1"/>
+    <row r="95" ht="15" customHeight="1"/>
+    <row r="96" ht="15" customHeight="1"/>
+    <row r="97" ht="15" customHeight="1"/>
+    <row r="98" ht="15" customHeight="1"/>
+    <row r="99" ht="15" customHeight="1"/>
+    <row r="100" ht="15" customHeight="1"/>
+    <row r="101" ht="15" customHeight="1"/>
+    <row r="102" ht="15" customHeight="1"/>
+    <row r="103" ht="15" customHeight="1"/>
+    <row r="104" ht="15" customHeight="1"/>
+    <row r="105" ht="15" customHeight="1"/>
+    <row r="106" ht="15" customHeight="1"/>
+    <row r="107" ht="15" customHeight="1"/>
+    <row r="108" ht="15" customHeight="1"/>
+    <row r="109" ht="15" customHeight="1"/>
+    <row r="110" ht="15" customHeight="1"/>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A20:B20"/>
+  <mergeCells count="7">
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A9:B9"/>
   </mergeCells>
   <hyperlinks>
@@ -7549,7 +7186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7563,103 +7200,100 @@
           <t>INST-BR-02 — Pobieranie przy zerowych wynikach generuje pusty plik XLSX bez nagłówka</t>
         </is>
       </c>
-      <c r="B1" s="18" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Metadane</t>
         </is>
       </c>
-      <c r="B2" s="20" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B3" s="22" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>INST-BR-02</t>
         </is>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Tytuł</t>
         </is>
       </c>
-      <c r="B4" s="22" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Pobieranie przy zerowych wynikach generuje pusty plik XLSX bez nagłówka</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Priorytet</t>
         </is>
       </c>
-      <c r="B5" s="30" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>P3 · Niski</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Ważność/dotkliwość</t>
         </is>
       </c>
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>Niska</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Powiązany scenariusz testowy</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>INST-17</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Data zgłoszenia</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Środowisko</t>
         </is>
       </c>
-      <c r="B9" s="20" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7674,56 +7308,55 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Przeglądarka</t>
         </is>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Chrome 151</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>System operacyjny</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>macOS 15.7.4</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Rozdzielczość</t>
         </is>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>1440×900</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Reprodukcja</t>
         </is>
       </c>
-      <c r="B14" s="20" t="n"/>
     </row>
     <row r="15" ht="112" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Kroki reprodukcji</t>
         </is>
       </c>
-      <c r="B15" s="22" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7799,13 +7432,20 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Rezultat</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Oczekiwany rezultat</t>
         </is>
       </c>
-      <c r="B16" s="25" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7832,13 +7472,13 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Rzeczywisty rezultat</t>
         </is>
       </c>
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7880,21 +7520,20 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="19" t="inlineStr">
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Analiza wpływu</t>
         </is>
       </c>
-      <c r="B18" s="20" t="n"/>
-    </row>
-    <row r="19" ht="64" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
+    </row>
+    <row r="20" ht="64" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Wpływ na użytkownika</t>
         </is>
       </c>
-      <c r="B19" s="22" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7921,129 +7560,48 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="19" t="inlineStr">
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>Załączniki</t>
         </is>
       </c>
-      <c r="B20" s="20" t="n"/>
-    </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="27" t="n"/>
-      <c r="B21" s="20" t="n"/>
-    </row>
-    <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="27" t="n"/>
-      <c r="B22" s="20" t="n"/>
-    </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="27" t="n"/>
-      <c r="B23" s="20" t="n"/>
-    </row>
-    <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="27" t="n"/>
-      <c r="B24" s="20" t="n"/>
-    </row>
-    <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="27" t="n"/>
-      <c r="B25" s="20" t="n"/>
-    </row>
-    <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="27" t="n"/>
-      <c r="B26" s="20" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="27" t="n"/>
-      <c r="B27" s="20" t="n"/>
-    </row>
-    <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="27" t="n"/>
-      <c r="B28" s="20" t="n"/>
-    </row>
-    <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="27" t="n"/>
-      <c r="B29" s="20" t="n"/>
-    </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="27" t="n"/>
-      <c r="B30" s="20" t="n"/>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="27" t="n"/>
-      <c r="B31" s="20" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="27" t="n"/>
-      <c r="B32" s="20" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="27" t="n"/>
-      <c r="B33" s="20" t="n"/>
-    </row>
-    <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="27" t="n"/>
-      <c r="B34" s="20" t="n"/>
-    </row>
-    <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="27" t="n"/>
-      <c r="B35" s="20" t="n"/>
-    </row>
-    <row r="36" ht="15" customHeight="1">
-      <c r="A36" s="27" t="n"/>
-      <c r="B36" s="20" t="n"/>
-    </row>
-    <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="27" t="n"/>
-      <c r="B37" s="20" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="27" t="n"/>
-      <c r="B38" s="20" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="27" t="n"/>
-      <c r="B39" s="20" t="n"/>
-    </row>
-    <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="27" t="n"/>
-      <c r="B40" s="20" t="n"/>
-    </row>
-    <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="27" t="n"/>
-      <c r="B41" s="20" t="n"/>
-    </row>
-    <row r="42" ht="15" customHeight="1">
-      <c r="A42" s="27" t="n"/>
-      <c r="B42" s="20" t="n"/>
-    </row>
-    <row r="43" ht="15" customHeight="1">
-      <c r="A43" s="27" t="n"/>
-      <c r="B43" s="20" t="n"/>
-    </row>
-    <row r="44" ht="15" customHeight="1">
-      <c r="A44" s="27" t="n"/>
-      <c r="B44" s="20" t="n"/>
-    </row>
-    <row r="45" ht="15" customHeight="1">
-      <c r="A45" s="27" t="n"/>
-      <c r="B45" s="20" t="n"/>
-    </row>
-    <row r="46" ht="15" customHeight="1">
-      <c r="A46" s="27" t="n"/>
-      <c r="B46" s="20" t="n"/>
-    </row>
-    <row r="47" ht="15" customHeight="1">
-      <c r="A47" s="28" t="n"/>
-      <c r="B47" s="29" t="n"/>
-    </row>
+    </row>
+    <row r="22" ht="15" customHeight="1"/>
+    <row r="23" ht="15" customHeight="1"/>
+    <row r="24" ht="15" customHeight="1"/>
+    <row r="25" ht="15" customHeight="1"/>
+    <row r="26" ht="15" customHeight="1"/>
+    <row r="27" ht="15" customHeight="1"/>
+    <row r="28" ht="15" customHeight="1"/>
+    <row r="29" ht="15" customHeight="1"/>
+    <row r="30" ht="15" customHeight="1"/>
+    <row r="31" ht="15" customHeight="1"/>
+    <row r="32" ht="15" customHeight="1"/>
+    <row r="33" ht="15" customHeight="1"/>
+    <row r="34" ht="15" customHeight="1"/>
+    <row r="35" ht="15" customHeight="1"/>
+    <row r="36" ht="15" customHeight="1"/>
+    <row r="37" ht="15" customHeight="1"/>
+    <row r="38" ht="15" customHeight="1"/>
+    <row r="39" ht="15" customHeight="1"/>
+    <row r="40" ht="15" customHeight="1"/>
+    <row r="41" ht="15" customHeight="1"/>
+    <row r="42" ht="15" customHeight="1"/>
+    <row r="43" ht="15" customHeight="1"/>
+    <row r="44" ht="15" customHeight="1"/>
+    <row r="45" ht="15" customHeight="1"/>
+    <row r="46" ht="15" customHeight="1"/>
+    <row r="47" ht="15" customHeight="1"/>
+    <row r="48" ht="15" customHeight="1"/>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A20:B20"/>
+  <mergeCells count="7">
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A9:B9"/>
   </mergeCells>
   <hyperlinks>

</xml_diff>

<commit_message>
fix(/qa-case): proper internal sheet hyperlinks via Hyperlink(location=...)
Poprzednie użycie cell.hyperlink = "#'Sheet'!A1" generowało w XLSX XML
external file link:
  <Relationship Target="#'Test cases'!A8" TargetMode="External"/>

Excel/Numbers próbował otworzyć plik o nazwie "#'Test cases'!A8" i zgłaszał
"Łącze jest nieprawidłowe".

Fix: użyj openpyxl.worksheet.hyperlink.Hyperlink object z location=
parameter zamiast string cell.hyperlink. Produkuje właściwy XML:
  <hyperlink ref="B7" location="'Test cases'!A8" display="INST-07"/>

Excel, Numbers i Google Sheets rozpoznają to jako internal sheet jump.
Brak external Target/TargetMode w rels file.

Zastosowane w add_bug_id_hyperlinks() dla obu kierunków:
- Test cases "ID buga" -> bug tab
- Bug tab "Powiązany scenariusz testowy" -> Test cases row

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
+++ b/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
@@ -4991,8 +4991,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId2"/>
+    <hyperlink ref="I8" location="'INST-BR-01'!A1" display="INST-BR-01"/>
+    <hyperlink ref="I18" location="'INST-BR-02'!A1" display="INST-BR-02"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7172,10 +7172,10 @@
     <mergeCell ref="A9:B9"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
+    <hyperlink ref="B7" location="'Test cases'!A8" display="INST-07"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7605,9 +7605,9 @@
     <mergeCell ref="A9:B9"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
+    <hyperlink ref="B7" location="'Test cases'!A18" display="INST-17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(/qa-case): usun Execution report zakladke z XLSX (redundant z bug tabs)
Analiza duplikacji Execution report:
- ID + Status + Wynik: juz w Test cases (Wynik column mirroruje Status)
- Rzeczywisty rezultat + Waga + Zrzut ekranu + Reprodukcja: dla FAIL
  cases juz w dedykowanych bug tabs (INST-BR-XX) w bogatszym ukladzie
  (embedded screenshot, sekcje, color-coded)
- Dla PASS cases: wszystkie wartosci to "-" (bezwartościowe)

Fix: skip generacji Execution report zakladki w XLSX. Plik -report.tsv
zostaje jako aggregated backup source (git diff, potencjalna regeneracja).

Zmiany:
- scripts/qa-tsv-to-xlsx.py: skip create_sheet("Execution report")
- SKILL.md pkt 1 (Output): zakladki teraz "Test cases + N zakladek per-bug"
  (bez Execution report)
- SKILL.md pkt 4 (-report.tsv): "aggregated data source, NIE renderuje sie
  jako zakladka XLSX"

XLSX ma teraz 3 zakladki zamiast 4: Test cases + INST-BR-01 + INST-BR-02.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
+++ b/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
@@ -8,9 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution report" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INST-BR-01" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INST-BR-02" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INST-BR-01" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INST-BR-02" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -208,12 +207,6 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -223,6 +216,9 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -231,6 +227,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5001,1599 +5000,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00305496"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Rzeczywisty rezultat</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Waga</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Zrzut ekranu</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Reprodukcja</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>INST-01</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Vistula → Znaleziono: 22, pierwszy wiersz: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Akademia Finansów i Biznesu Vistula"</t>
-          </r>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>INST-02</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Link </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Akademia Finansów i Biznesu Vistula"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> ma target=</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"_blank"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">, href </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="FF0563C1"/>
-              <sz val="10"/>
-              <u val="single"/>
-            </rPr>
-            <t>/wyszukiwarka-instytucji/instytucje/Akademia-Finans</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>%C3%B3w-i-Biznesu-Vistula,30170</t>
-          </r>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>INST-03</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Link </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"http://www.vistula.edu.pl/"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> na stronie detali ma target=</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"_blank"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> + rel=</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"noopener noreferrer"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> — bezpieczne otwarcie</t>
-          </r>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>INST-04</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Puste ?search= → licznik 2605 (pełna lista); URL po loadzie stripowany do ?limit=20&amp;offset=0</t>
-          </r>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>INST-05</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Fraza </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"nieistniejacax9y9z9qwerty"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> → Znaleziono: 0, tabela </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Brak danych"</t>
-          </r>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>INST-06</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">łódź=84, ŁÓDŹ=84 (wielkość liter ignorowana); </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"  Vistula  "</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> (z spacjami) = Vistula = 22 (spacje na krańcach przycięte); Filia; = 204 (średnik jako znak specjalny nie łamie wyszukiwania)</t>
-          </r>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>INST-07</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">lodz (bez ogonków) → Znaleziono: 1; </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"łódź"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> (z ogonkami) → Znaleziono: 84. Backend nie wykonuje asciifolding / unaccent — użytkownik piszący </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"lodz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> traci 83 wyniki, które faktycznie zawierają </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Łódź"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> w nazwie</t>
-          </r>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>Średnia</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>qa-runs/screenshots/INST-07.png</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">1) Otwórz </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="FF0563C1"/>
-              <sz val="10"/>
-              <u val="single"/>
-            </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-2) W pole wyszukiwania wpisz frazę </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"lodz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> (bez polskich znaków / bez ogonków)
-3) Poczekaj ~2–3s i zapisz licznik </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Znaleziono"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-4) Wyczyść pole (Cmd</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="FF0563C1"/>
-              <sz val="10"/>
-              <u val="single"/>
-            </rPr>
-            <t>/Ctrl</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">+A + Delete), wpisz </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"łódź"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> (z polskimi znakami), poczekaj i zapisz licznik referencyjny (~84)
-5) Porównaj oba liczniki</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>INST-08</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">500-char query </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"a…"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> → 0 wyników, </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Brak danych"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">, brak crashu. XSS payload </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"&lt;script&gt;alert(1)&lt;/script&gt;"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> wyrenderowany jako tekst, brak execution, brak &lt;script&gt; w DOM. limit=abc normalizowany na 20, offset=-1 na -20 (dziwna normalizacja, ale bez crashu i stack trace)</t>
-          </r>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>INST-09</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>IC checkbox → licznik 2605→579, URL &amp;roles=1</t>
-          </r>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>INST-10</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>wolnorynkowe checkbox → licznik 2605→202, URL &amp;qualification_categories=5</t>
-          </r>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>INST-11</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Combobox Siedziba </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Warszawa"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> → licznik 2605→350, URL &amp;cities=Warszawa</t>
-          </r>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>INST-12</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>roles=1 + qualification_categories=5 → licznik 148 (&lt; min(579, 202) = 202), AND logic potwierdzona</t>
-          </r>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>INST-13</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Klik ikony (i) obok </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Zadania w ZSK"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> otworzył modal role=dialog z nagłówkiem </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Pomoc"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> i treścią: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Instytucja certyfikująca (IC) – uprawniona instytucja…"</t>
-          </r>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>INST-14</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">search=nieistniejaca_instytucja_xyz + roles=1 → Znaleziono: 0, </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Brak danych"</t>
-          </r>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>INST-15</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Pobierz z ?search=Vistula → plik lista_instytucji.xlsx, 23 wierszy (header + 22 danych), zgodne z licznikiem 22</t>
-          </r>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>INST-16</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Pobierz bez filtrów → plik lista_instytucji.xlsx, 2606 wierszy (header + 2605 danych), zgodne z licznikiem 2605</t>
-          </r>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>INST-17</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Przycisk </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Pobierz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> nie jest disabled przy licznikiku 0. Pobrany plik ma 1 wiersz × 1 kolumnę, komórka = None (pusty XLSX bez nawet nagłówka </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"#/ID/Nazwa"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>Niska</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>qa-runs/screenshots/INST-17.png</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">1) Otwórz </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="FF0563C1"/>
-              <sz val="10"/>
-              <u val="single"/>
-            </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-2) W pole wyszukiwania wpisz frazę </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"nieistniejaca_xyz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> i poczekaj aż licznik pokaże </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Znaleziono: 0"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-3) Kliknij przycisk </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Pobierz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-4) Otwórz pobrany plik i sprawdź czy zawiera nagłówek kolumn</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>INST-18</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Klik Next na offset=0 → URL ?limit=20&amp;offset=20, info paginacji </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"21–40 z 2605"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>, tabela pokazała nowe wiersze</t>
-          </r>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>INST-19</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Na offset=0 przycisk </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Go to previous page"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> ma disabled=true</t>
-          </r>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>INST-20</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Na offset=2600 przycisk </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Go to next page"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> ma disabled=true, info paginacji </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"2601–2605 z 2605"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>, tabela pokazała 5 wierszy</t>
-          </r>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>INST-21</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Na wszystkich 3 rozmiarach okna (1280×720, 1440×900, 1920×1080): brak paska przewijania poziomego na dole okna, core UI (pole wyszukiwania, filtry, tabela wyników) w pełni widoczne bez ucinania</t>
-          </r>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>INST-22</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Okno 768×1024: brak paska przewijania poziomego, filtry i tabela wyników widoczne bez ucinania</t>
-          </r>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>INST-23</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Okno 375×812: brak paska przewijania poziomego, licznik </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Znaleziono"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> i tabela wyników widoczne bez ucinania</t>
-          </r>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>INST-24</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Wymaga wykonania manualnego przez testera (patrz Kroki w cases sheet)</t>
-          </r>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>INST-25</t>
-        </is>
-      </c>
-      <c r="B26" s="14" t="inlineStr">
-        <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Wymaga wykonania manualnego przez testera (patrz Kroki w cases sheet)</t>
-          </r>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>INST-26</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Wymaga wykonania manualnego przez testera (patrz Kroki w cases sheet)</t>
-          </r>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <tabColor rgb="00FFC000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -6607,21 +5013,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>INST-BR-01 — Wyszukiwarka nie znajduje polskich nazw gdy fraza wpisana bez polskich znaków</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Metadane</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
@@ -6633,7 +5039,7 @@
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Tytuł</t>
         </is>
@@ -6645,43 +5051,43 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Priorytet</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>P2 · Wysoki</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Ważność/dotkliwość</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Średnia</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Powiązany scenariusz testowy</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>INST-07</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Data zgłoszenia</t>
         </is>
@@ -6693,14 +5099,14 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Środowisko</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -6720,7 +5126,7 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Przeglądarka</t>
         </is>
@@ -6732,7 +5138,7 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>System operacyjny</t>
         </is>
@@ -6744,7 +5150,7 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Rozdzielczość</t>
         </is>
@@ -6756,14 +5162,14 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Reprodukcja</t>
         </is>
       </c>
     </row>
     <row r="15" ht="144" customHeight="1">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Kroki reprodukcji</t>
         </is>
@@ -6862,19 +5268,19 @@
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Rezultat</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Oczekiwany rezultat</t>
         </is>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6955,12 +5361,12 @@
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Rzeczywisty rezultat</t>
         </is>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7026,14 +5432,14 @@
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Analiza wpływu</t>
         </is>
       </c>
     </row>
     <row r="20" ht="80" customHeight="1">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Wpływ na użytkownika</t>
         </is>
@@ -7066,7 +5472,7 @@
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Załączniki</t>
         </is>
@@ -7179,7 +5585,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00A6A6A6"/>
@@ -7195,21 +5601,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>INST-BR-02 — Pobieranie przy zerowych wynikach generuje pusty plik XLSX bez nagłówka</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Metadane</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
@@ -7221,7 +5627,7 @@
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Tytuł</t>
         </is>
@@ -7233,43 +5639,43 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Priorytet</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>P3 · Niski</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Ważność/dotkliwość</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Niska</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Powiązany scenariusz testowy</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>INST-17</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Data zgłoszenia</t>
         </is>
@@ -7281,14 +5687,14 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Środowisko</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -7308,7 +5714,7 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Przeglądarka</t>
         </is>
@@ -7320,7 +5726,7 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>System operacyjny</t>
         </is>
@@ -7332,7 +5738,7 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Rozdzielczość</t>
         </is>
@@ -7344,14 +5750,14 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Reprodukcja</t>
         </is>
       </c>
     </row>
     <row r="15" ht="112" customHeight="1">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Kroki reprodukcji</t>
         </is>
@@ -7433,19 +5839,19 @@
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Rezultat</t>
         </is>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Oczekiwany rezultat</t>
         </is>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7473,12 +5879,12 @@
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Rzeczywisty rezultat</t>
         </is>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -7521,14 +5927,14 @@
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Analiza wpływu</t>
         </is>
       </c>
     </row>
     <row r="20" ht="64" customHeight="1">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Wpływ na użytkownika</t>
         </is>
@@ -7561,7 +5967,7 @@
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Załączniki</t>
         </is>

</xml_diff>

<commit_message>
chore: zebrane zmiany z poprzednich sesji (INST run, scripts, screenshots)
- .gitignore: dodane .DS_Store patterns
- wyszukiwarka-instytucji-2026-08-15-*: aktualizacje run-u (bugs.tsv, cases.tsv,
  report.tsv, .md, .xlsx) + usunięcie INST-BR-02.md (bug wycofany)
  + qa-runs/screenshots/INST-13.png (dołączony do run-u)
- scripts/generate-notes-pdf.js, reorganize-notes.js — helpery do notatek
  interviewowych
- scripts/two-user-chat-loadgen.js — load generator dla PhoneHQ chat testów
- Screenshots w repo root:
  - bug1-ksiegowy-no-results.png, bug2-dziedzina-no-label-viewport.png
    (screenshots z zadania kwalifikacji, wersja alt vs qa-task-kwalifikacje/)
  - ens-*.png (8x) — screenshots z ENS run

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
+++ b/qa-runs/wyszukiwarka-instytucji-2026-08-15.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INST-BR-01" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INST-BR-02" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -74,7 +73,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -109,11 +108,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -163,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -201,16 +195,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -222,14 +213,11 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -317,36 +305,6 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="6191250" cy="12668250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>21</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6191250" cy="3867150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -657,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3581,12 +3539,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Pobieranie przy zerowych wynikach nie generuje pustego pliku bez nagłówka</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
-        <is>
-          <t>P3 · Niski</t>
+          <t>Przycisk Następna strona przechodzi do kolejnych 20 wyników</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>P1 · Krytyczny</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -3596,7 +3554,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Wyszukiwarka z frazą bez dopasowań (licznik = 0)</t>
+            <t>Wyszukiwarka na stronie 1 (offset=0), Next enabled</t>
           </r>
         </is>
       </c>
@@ -3607,22 +3565,15 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">fraza: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"nieistniejaca_xyz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>, licznik = 0</t>
+            <t xml:space="preserve">Kliknięcie </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Go to next page"</t>
           </r>
         </is>
       </c>
@@ -3642,7 +3593,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0</t>
           </r>
           <r>
             <rPr>
@@ -3650,30 +3601,31 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) W pole wyszukiwania wpisz frazę </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"nieistniejaca_xyz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> i poczekaj aż licznik pokaże </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Znaleziono: 0"</t>
+2) Zapisz info paginacji (np. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"1–20 z 2605"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">)
+3) Kliknij przycisk paginacji </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Go to next page"</t>
           </r>
           <r>
             <rPr>
@@ -3681,23 +3633,7 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-3) Kliknij przycisk </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Pobierz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-4) Otwórz pobrany plik i sprawdź czy zawiera nagłówek kolumn</t>
+4) Sprawdź URL i info</t>
           </r>
         </is>
       </c>
@@ -3708,38 +3644,53 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">Przycisk </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Pobierz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> jest wyłączony LUB pobrany plik zawiera co najmniej nagłówek kolumn (nie tylko pusty arkusz)</t>
-          </r>
-        </is>
-      </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="I18" s="12" t="inlineStr">
-        <is>
-          <t>INST-BR-02</t>
-        </is>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>Przycisk nie jest disabled, plik ma 1×1 arkusz z pustą komórką (brak nawet nagłówka "#/ID/Nazwa") — mylące dla usera</t>
+            <t xml:space="preserve">URL zawiera </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"&amp;offset=20"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">, info paginacji: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"21–40 z 2605"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t>, tabela pokazuje nowe wiersze</t>
+          </r>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -3751,12 +3702,12 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Przycisk Następna strona przechodzi do kolejnych 20 wyników</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>P1 · Krytyczny</t>
+          <t>Na pierwszej stronie przycisk Poprzednia jest wyłączony</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>P2 · Wysoki</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -3766,7 +3717,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Wyszukiwarka na stronie 1 (offset=0), Next enabled</t>
+            <t>Wyszukiwarka na stronie 1 (offset=0)</t>
           </r>
         </is>
       </c>
@@ -3777,15 +3728,15 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">Kliknięcie </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Go to next page"</t>
+            <t xml:space="preserve">stan przycisku </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Go to previous page"</t>
           </r>
         </is>
       </c>
@@ -3813,39 +3764,15 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Zapisz info paginacji (np. </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"1–20 z 2605"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">)
-3) Kliknij przycisk paginacji </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Go to next page"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-4) Sprawdź URL i info</t>
+2) Zbadaj atrybut disabled przycisku </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Go to previous page"</t>
           </r>
         </is>
       </c>
@@ -3856,37 +3783,22 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">URL zawiera </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"&amp;offset=20"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">, info paginacji: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"21–40 z 2605"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>, tabela pokazuje nowe wiersze</t>
+            <t xml:space="preserve">Przycisk </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Poprzednia"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> ma disabled=true, klik nie ma efektu</t>
           </r>
         </is>
       </c>
@@ -3914,7 +3826,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Na pierwszej stronie przycisk Poprzednia jest wyłączony</t>
+          <t>Na ostatniej stronie przycisk Następna jest wyłączony</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -3929,7 +3841,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Wyszukiwarka na stronie 1 (offset=0)</t>
+            <t>Wyszukiwarka na ostatniej stronie (offset=2600, 2601–2605)</t>
           </r>
         </is>
       </c>
@@ -3948,7 +3860,7 @@
               <b val="1"/>
               <sz val="10"/>
             </rPr>
-            <t>"Go to previous page"</t>
+            <t>"Go to next page"</t>
           </r>
         </is>
       </c>
@@ -3968,7 +3880,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=0</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=2600</t>
           </r>
           <r>
             <rPr>
@@ -3984,7 +3896,7 @@
               <b val="1"/>
               <sz val="10"/>
             </rPr>
-            <t>"Go to previous page"</t>
+            <t>"Go to next page"</t>
           </r>
         </is>
       </c>
@@ -4003,14 +3915,29 @@
               <b val="1"/>
               <sz val="10"/>
             </rPr>
-            <t>"Poprzednia"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> ma disabled=true, klik nie ma efektu</t>
+            <t>"Następna"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> ma disabled=true, info paginacji: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"2601–2605 z 2605"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t>, tabela pokazuje 5 wierszy</t>
           </r>
         </is>
       </c>
@@ -4024,9 +3951,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>URL ?offset=2600 jako skrót do stanu „ostatnia strona"; interakcja Next pokryta w INST-18</t>
         </is>
       </c>
     </row>
@@ -4038,12 +3965,12 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Na ostatniej stronie przycisk Następna jest wyłączony</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>P2 · Wysoki</t>
+          <t>Wyszukiwarka renderuje się poprawnie na typowych rozdzielczościach desktop</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>P1 · Krytyczny</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
@@ -4053,7 +3980,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Wyszukiwarka na ostatniej stronie (offset=2600, 2601–2605)</t>
+            <t>Przeglądarka desktopowa z możliwością zmiany rozmiaru okna (DevTools lub natywnie)</t>
           </r>
         </is>
       </c>
@@ -4064,15 +3991,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">stan przycisku </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Go to next page"</t>
+            <t>viewporty testowane: 1280×720 (małe laptopy, dolny próg), 1440×900 (MBP default), 1920×1080 (FHD monitor)</t>
           </r>
         </is>
       </c>
@@ -4083,7 +4002,23 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">1) Otwórz </t>
+            <t xml:space="preserve">1) Ustaw okno przeglądarki na rozmiar 1280×720 pikseli (DevTools → Toggle device toolbar → wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"1280 × 720"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> w polach szerokość × wysokość)
+2) Otwórz </t>
           </r>
           <r>
             <rPr>
@@ -4092,7 +4027,7 @@
               <sz val="10"/>
               <u val="single"/>
             </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/?limit=20&amp;offset=2600</t>
+            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
           </r>
           <r>
             <rPr>
@@ -4100,15 +4035,24 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-2) Zbadaj atrybut disabled przycisku </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Go to next page"</t>
+3) Poczekaj ~2s na załadowanie strony i sprawdź wzrokowo: (a) NIE ma poziomego paska przewijania na dole okna, (b) widoczne w całości bez ucinania: pole wyszukiwania, sekcje filtrów, licznik </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Znaleziono"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t>, tabela wyników
+4) Powtórz kroki 1–3 dla rozmiaru okna 1440×900
+5) Powtórz kroki 1–3 dla rozmiaru okna 1920×1080</t>
           </r>
         </is>
       </c>
@@ -4119,37 +4063,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">Przycisk </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Następna"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> ma disabled=true, info paginacji: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"2601–2605 z 2605"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>, tabela pokazuje 5 wierszy</t>
+            <t>Na każdym z 3 rozmiarów okna (1280×720, 1440×900, 1920×1080): brak poziomego paska przewijania na dole okna, wszystkie elementy wyszukiwarki (pole wyszukiwania, filtry, tabela) widoczne w pełni bez ucinania przez prawą krawędź</t>
           </r>
         </is>
       </c>
@@ -4165,7 +4079,7 @@
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>URL ?offset=2600 jako skrót do stanu „ostatnia strona"; interakcja Next pokryta w INST-18</t>
+          <t>Zaobserwowano: brak paska przewijania poziomego i pełną widoczność core UI na wszystkich 3 rozmiarach okna (1280×720, 1440×900, 1920×1080)</t>
         </is>
       </c>
     </row>
@@ -4177,7 +4091,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Wyszukiwarka renderuje się poprawnie na typowych rozdzielczościach desktop</t>
+          <t>Wyszukiwarka mieści się w ekranie tabletu bez poziomego przewijania</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -4192,7 +4106,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Przeglądarka desktopowa z możliwością zmiany rozmiaru okna (DevTools lub natywnie)</t>
+            <t>Viewport 768×1024 px</t>
           </r>
         </is>
       </c>
@@ -4203,7 +4117,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>viewporty testowane: 1280×720 (małe laptopy, dolny próg), 1440×900 (MBP default), 1920×1080 (FHD monitor)</t>
+            <t>viewport: 768×1024</t>
           </r>
         </is>
       </c>
@@ -4214,22 +4128,37 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">1) Ustaw okno przeglądarki na rozmiar 1280×720 pikseli (DevTools → Toggle device toolbar → wpisz </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"1280 × 720"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> w polach szerokość × wysokość)
+            <t xml:space="preserve">1) Ustaw okno przeglądarki na rozmiar 768×1024 pikseli (DevTools → Toggle device toolbar → wybierz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"iPad"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> LUB wpisz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"768 × 1024"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">)
 2) Otwórz </t>
           </r>
           <r>
@@ -4247,24 +4176,8 @@
               <sz val="10"/>
             </rPr>
             <t xml:space="preserve">
-3) Poczekaj ~2s na załadowanie strony i sprawdź wzrokowo: (a) NIE ma poziomego paska przewijania na dole okna, (b) widoczne w całości bez ucinania: pole wyszukiwania, sekcje filtrów, licznik </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Znaleziono"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>, tabela wyników
-4) Powtórz kroki 1–3 dla rozmiaru okna 1440×900
-5) Powtórz kroki 1–3 dla rozmiaru okna 1920×1080</t>
+3) Poczekaj ~2s na załadowanie strony
+4) Sprawdź wzrokowo: brak poziomego paska przewijania na dole okna, widoczne pole wyszukiwania, sekcje filtrów i tabela wyników bez ucinania</t>
           </r>
         </is>
       </c>
@@ -4275,7 +4188,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Na każdym z 3 rozmiarów okna (1280×720, 1440×900, 1920×1080): brak poziomego paska przewijania na dole okna, wszystkie elementy wyszukiwarki (pole wyszukiwania, filtry, tabela) widoczne w pełni bez ucinania przez prawą krawędź</t>
+            <t>Brak poziomego paska przewijania na dole okna, filtry i tabela wyników widoczne bez ucinania</t>
           </r>
         </is>
       </c>
@@ -4291,7 +4204,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Zaobserwowano: brak paska przewijania poziomego i pełną widoczność core UI na wszystkich 3 rozmiarach okna (1280×720, 1440×900, 1920×1080)</t>
+          <t>Zaobserwowano: brak paska przewijania poziomego na tablecie 768×1024, wszystkie elementy widoczne</t>
         </is>
       </c>
     </row>
@@ -4303,7 +4216,7 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Wyszukiwarka mieści się w ekranie tabletu bez poziomego przewijania</t>
+          <t>Wyszukiwarka mieści się w ekranie telefonu bez poziomego przewijania</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -4318,7 +4231,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Viewport 768×1024 px</t>
+            <t>Viewport 375×812 px</t>
           </r>
         </is>
       </c>
@@ -4329,7 +4242,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>viewport: 768×1024</t>
+            <t>viewport: 375×812</t>
           </r>
         </is>
       </c>
@@ -4340,15 +4253,30 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">1) Ustaw okno przeglądarki na rozmiar 768×1024 pikseli (DevTools → Toggle device toolbar → wybierz </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"iPad"</t>
+            <t xml:space="preserve">1) Ustaw okno przeglądarki na rozmiar 375×812 pikseli (DevTools → Toggle device toolbar → wybierz </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"iPhone SE"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> lub </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"iPhone 12/13"</t>
           </r>
           <r>
             <rPr>
@@ -4363,7 +4291,7 @@
               <b val="1"/>
               <sz val="10"/>
             </rPr>
-            <t>"768 × 1024"</t>
+            <t>"375 × 812"</t>
           </r>
           <r>
             <rPr>
@@ -4389,7 +4317,7 @@
             </rPr>
             <t xml:space="preserve">
 3) Poczekaj ~2s na załadowanie strony
-4) Sprawdź wzrokowo: brak poziomego paska przewijania na dole okna, widoczne pole wyszukiwania, sekcje filtrów i tabela wyników bez ucinania</t>
+4) Sprawdź wzrokowo: brak poziomego paska przewijania na dole okna, core flow (pole wyszukiwania + filtry + tabela) widoczny bez ucinania</t>
           </r>
         </is>
       </c>
@@ -4400,7 +4328,22 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Brak poziomego paska przewijania na dole okna, filtry i tabela wyników widoczne bez ucinania</t>
+            <t xml:space="preserve">Brak poziomego paska przewijania na dole okna, licznik </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>"Znaleziono"</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve"> i tabela wyników widoczne bez ucinania</t>
           </r>
         </is>
       </c>
@@ -4416,7 +4359,7 @@
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>Zaobserwowano: brak paska przewijania poziomego na tablecie 768×1024, wszystkie elementy widoczne</t>
+          <t>Zaobserwowano: brak paska przewijania poziomego na telefonie 375×812, wszystkie elementy widoczne</t>
         </is>
       </c>
     </row>
@@ -4428,7 +4371,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Wyszukiwarka mieści się w ekranie telefonu bez poziomego przewijania</t>
+          <t>Dostępność WCAG 2.2 AA — czytelność treści</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -4443,7 +4386,7 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>Viewport 375×812 px</t>
+            <t>axe DevTools zainstalowany, Chrome DevTools z Rendering panel</t>
           </r>
         </is>
       </c>
@@ -4454,166 +4397,11 @@
               <rFont val="Calibri"/>
               <sz val="10"/>
             </rPr>
-            <t>viewport: 375×812</t>
+            <t>strona bazowa + strona detali instytucji</t>
           </r>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">1) Ustaw okno przeglądarki na rozmiar 375×812 pikseli (DevTools → Toggle device toolbar → wybierz </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"iPhone SE"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> lub </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"iPhone 12/13"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> LUB wpisz </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"375 × 812"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">)
-2) Otwórz </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="FF0563C1"/>
-              <sz val="10"/>
-              <u val="single"/>
-            </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-3) Poczekaj ~2s na załadowanie strony
-4) Sprawdź wzrokowo: brak poziomego paska przewijania na dole okna, core flow (pole wyszukiwania + filtry + tabela) widoczny bez ucinania</t>
-          </r>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Brak poziomego paska przewijania na dole okna, licznik </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Znaleziono"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> i tabela wyników widoczne bez ucinania</t>
-          </r>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>Zaobserwowano: brak paska przewijania poziomego na telefonie 375×812, wszystkie elementy widoczne</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>INST-24</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Dostępność WCAG 2.2 AA — czytelność treści</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>P1 · Krytyczny</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>axe DevTools zainstalowany, Chrome DevTools z Rendering panel</t>
-          </r>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>strona bazowa + strona detali instytucji</t>
-          </r>
-        </is>
-      </c>
-      <c r="F25" s="9" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4660,7 +4448,7 @@
           </r>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4671,39 +4459,39 @@
           </r>
         </is>
       </c>
-      <c r="H25" s="14" t="inlineStr">
+      <c r="H24" s="13" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J25" s="9" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>Wymaga manualnej weryfikacji przez testera. ~30 min. Krytyczne dla portalu .gov.pl (Ustawa o dostępności cyfrowej)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>INST-25</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>INST-24</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Dostępność WCAG 2.2 AA — pełna obsługa z klawiatury</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>P1 · Krytyczny</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4714,7 +4502,7 @@
           </r>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4725,7 +4513,7 @@
           </r>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4804,7 +4592,7 @@
           </r>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4815,39 +4603,39 @@
           </r>
         </is>
       </c>
-      <c r="H26" s="14" t="inlineStr">
+      <c r="H25" s="13" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J26" s="5" t="inlineStr">
+      <c r="J25" s="9" t="inlineStr">
         <is>
           <t>Wymaga manualnej weryfikacji przez testera. ~45 min. Krytyczne dla portalu .gov.pl</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>INST-26</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>INST-25</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Dostępność WCAG 2.2 AA — zrozumiałość i technologie wspomagające</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>P1 · Krytyczny</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4858,7 +4646,7 @@
           </r>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4869,7 +4657,7 @@
           </r>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4946,7 +4734,7 @@
           </r>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4972,17 +4760,17 @@
           </r>
         </is>
       </c>
-      <c r="H27" s="14" t="inlineStr">
+      <c r="H26" s="13" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J27" s="9" t="inlineStr">
+      <c r="J26" s="5" t="inlineStr">
         <is>
           <t>Wymaga manualnej weryfikacji przez testera. ~30 min. Znany bug pokrewny w wyszukiwarce kwalifikacji (BR-02: search input bez aria-label) — sprawdź czy dotyczy też tej wyszukiwarki</t>
         </is>
@@ -4991,7 +4779,6 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="I8" location="'INST-BR-01'!A1" display="INST-BR-01"/>
-    <hyperlink ref="I18" location="'INST-BR-02'!A1" display="INST-BR-02"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5013,21 +4800,21 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>INST-BR-01 — Wyszukiwarka nie znajduje polskich nazw gdy fraza wpisana bez polskich znaków</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>Metadane</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
@@ -5039,7 +4826,7 @@
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Tytuł</t>
         </is>
@@ -5051,43 +4838,43 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Priorytet</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>P2 · Wysoki</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Ważność/dotkliwość</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Średnia</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Powiązany scenariusz testowy</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>INST-07</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Data zgłoszenia</t>
         </is>
@@ -5099,14 +4886,14 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Środowisko</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
@@ -5126,7 +4913,7 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Przeglądarka</t>
         </is>
@@ -5138,7 +4925,7 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>System operacyjny</t>
         </is>
@@ -5150,7 +4937,7 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Rozdzielczość</t>
         </is>
@@ -5162,14 +4949,14 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Reprodukcja</t>
         </is>
       </c>
     </row>
     <row r="15" ht="144" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Kroki reprodukcji</t>
         </is>
@@ -5268,19 +5055,19 @@
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Rezultat</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Oczekiwany rezultat</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5361,12 +5148,12 @@
       </c>
     </row>
     <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Rzeczywisty rezultat</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5432,14 +5219,14 @@
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Analiza wpływu</t>
         </is>
       </c>
     </row>
     <row r="20" ht="80" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Wpływ na użytkownika</t>
         </is>
@@ -5472,7 +5259,7 @@
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Załączniki</t>
         </is>
@@ -5583,437 +5370,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00A6A6A6"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="85" customWidth="1" min="2" max="2"/>
-    <col hidden="1" width="13" customWidth="1" min="3" max="16384"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>INST-BR-02 — Pobieranie przy zerowych wynikach generuje pusty plik XLSX bez nagłówka</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="16" t="inlineStr">
-        <is>
-          <t>Metadane</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>INST-BR-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="17" t="inlineStr">
-        <is>
-          <t>Tytuł</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Pobieranie przy zerowych wynikach generuje pusty plik XLSX bez nagłówka</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>Priorytet</t>
-        </is>
-      </c>
-      <c r="B5" s="22" t="inlineStr">
-        <is>
-          <t>P3 · Niski</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Ważność/dotkliwość</t>
-        </is>
-      </c>
-      <c r="B6" s="22" t="inlineStr">
-        <is>
-          <t>Niska</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>Powiązany scenariusz testowy</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>INST-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Data zgłoszenia</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Środowisko</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="FF0563C1"/>
-              <sz val="10"/>
-              <u val="single"/>
-            </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>Przeglądarka</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Chrome 151</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>System operacyjny</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>macOS 15.7.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>Rozdzielczość</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>1440×900</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>Reprodukcja</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="112" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>Kroki reprodukcji</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">1) Otwórz </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="FF0563C1"/>
-              <sz val="10"/>
-              <u val="single"/>
-            </rPr>
-            <t>https://kwalifikacje.gov.pl/wyszukiwarka-instytucji/</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-2) W pole wyszukiwania wpisz frazę </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"nieistniejaca_xyz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> i poczekaj aż licznik pokaże </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Znaleziono: 0"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-3) Kliknij przycisk </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Pobierz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">
-4) Otwórz pobrany plik i sprawdź czy zawiera nagłówek kolumn</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>Rezultat</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Oczekiwany rezultat</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Przycisk </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Pobierz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> jest wyłączony LUB pobrany plik zawiera co najmniej nagłówek kolumn (nie tylko pusty arkusz)</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Rzeczywisty rezultat</t>
-        </is>
-      </c>
-      <c r="B18" s="21" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Przycisk </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Pobierz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> nie jest disabled przy liczniku 0. Pobrany plik ma 1 wiersz × 1 kolumnę, komórka = None (pusty XLSX bez nawet nagłówka </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"#/ID/Nazwa"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t>)</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>Analiza wpływu</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="64" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>Wpływ na użytkownika</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">Użytkownik przy pustym wyniku wyszukiwania klika </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>"Pobierz"</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> i dostaje niezrozumiały pusty plik zamiast informacji zwrotnej. Myślący że plik jest uszkodzony lub że eksport nie zadziałał. Rzadko trafia w flow (typowo user widzi 0 wyników i już nie pobiera), ale gdy trafi — mylące.</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>Załączniki</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1"/>
-    <row r="23" ht="15" customHeight="1"/>
-    <row r="24" ht="15" customHeight="1"/>
-    <row r="25" ht="15" customHeight="1"/>
-    <row r="26" ht="15" customHeight="1"/>
-    <row r="27" ht="15" customHeight="1"/>
-    <row r="28" ht="15" customHeight="1"/>
-    <row r="29" ht="15" customHeight="1"/>
-    <row r="30" ht="15" customHeight="1"/>
-    <row r="31" ht="15" customHeight="1"/>
-    <row r="32" ht="15" customHeight="1"/>
-    <row r="33" ht="15" customHeight="1"/>
-    <row r="34" ht="15" customHeight="1"/>
-    <row r="35" ht="15" customHeight="1"/>
-    <row r="36" ht="15" customHeight="1"/>
-    <row r="37" ht="15" customHeight="1"/>
-    <row r="38" ht="15" customHeight="1"/>
-    <row r="39" ht="15" customHeight="1"/>
-    <row r="40" ht="15" customHeight="1"/>
-    <row r="41" ht="15" customHeight="1"/>
-    <row r="42" ht="15" customHeight="1"/>
-    <row r="43" ht="15" customHeight="1"/>
-    <row r="44" ht="15" customHeight="1"/>
-    <row r="45" ht="15" customHeight="1"/>
-    <row r="46" ht="15" customHeight="1"/>
-    <row r="47" ht="15" customHeight="1"/>
-    <row r="48" ht="15" customHeight="1"/>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A9:B9"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="B7" location="'Test cases'!A18" display="INST-17"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>